<commit_message>
2026-05-22 docs: 주간보고 5/16~5/22 작성 + 개발현황 엑셀 갱신
- 주간보고: 본문 11개 항목 (운영 인프라 WS1~WS10·입출고 내역 2/3차·
  모바일 UI/UX 전면 개편 디자이너 PASS·불량 처리 흐름 재설계 Phase 1·
  BOM 워크벤치 3-column·권동환 5월 재고 100% 검증·CSV 외부 감시·
  ItemCode 도메인 정리·외부 PC 첫 실행·인수인계 문서·시스템 안정화)
- 추후 진행 예정 8개로 갱신 (BOM 동기화 우선·실 재고 입력·Wave3 보정·
  관리자 데스크톱·권한 연동·불량 Phase 2·인프라 백업/보안·외부 접근)
- generate_devlog.py: c10 추가, KPI 회사 기간 ~05-22 + 기능 완료 63/73,
  Sheet 2 5/16~5/22 행 추가 (5/9~5/15 완료 처리),
  features 9건 완료 + 1건(불량 Phase 2) 예정 추가
- 개발현황 엑셀 재생성 — 커밋 570건 · 근무 외 179건

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_attic/docs/개발현황.xlsx
+++ b/_attic/docs/개발현황.xlsx
@@ -619,7 +619,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -640,7 +640,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>2026-04-21 ~ 05-19 (회사 개발 착수 이후)</t>
+          <t>2026-04-21 ~ 05-22 (회사 개발 착수 이후)</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>536건 (회사 기간 448건)</t>
+          <t>570건 (회사 기간 490건)</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>55 / 64개 (86%)</t>
+          <t>63 / 73개 (86%)</t>
         </is>
       </c>
     </row>
@@ -1543,7 +1543,7 @@
               <color rgb="00000000"/>
               <sz val="10"/>
             </rPr>
-            <t>■</t>
+            <t>■■■■■■■■■■■■</t>
           </r>
           <r>
             <rPr>
@@ -1557,14 +1557,69 @@
               <color rgb="00000000"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">  (8)</t>
+            <t xml:space="preserve">  (30)</t>
           </r>
         </is>
       </c>
     </row>
+    <row r="39" ht="18" customHeight="1">
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">2026-05-21  </t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+              <sz val="10"/>
+            </rPr>
+            <t>■■■■■</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">  (11)</t>
+          </r>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">2026-05-22  </t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+              <sz val="10"/>
+            </rPr>
+            <t>■</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">  (1)</t>
+          </r>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="38">
+  <mergeCells count="40">
     <mergeCell ref="A30:E30"/>
+    <mergeCell ref="A39:E39"/>
     <mergeCell ref="A34:E34"/>
     <mergeCell ref="A24:E24"/>
     <mergeCell ref="A15:E15"/>
@@ -1601,6 +1656,7 @@
     <mergeCell ref="A19:E19"/>
     <mergeCell ref="A13:E13"/>
     <mergeCell ref="A31:E31"/>
+    <mergeCell ref="A40:E40"/>
     <mergeCell ref="A9:E9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1613,7 +1669,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1887,7 +1943,37 @@
       </c>
       <c r="E10" s="11" t="inlineStr">
         <is>
-          <t>진행 중</t>
+          <t>완료</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="60" customHeight="1">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-16 ~ 05-22</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>인프라·모바일·불량 처리</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>WS1~WS10 배포 안정화·보안 강화
+모바일 UI/UX 전면 개편(디자이너 PASS)
+불량 처리 흐름 재설계 Phase 1 (라인 결재·격리·처리)
+BOM 워크벤치 3-column·완료 워크플로
+입출고 내역 2·3차 main 머지
+권동환 5월 재고 100% 검증·CSV 외부 감시·ItemCode rename</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="n">
+        <v>127</v>
+      </c>
+      <c r="E11" s="11" t="inlineStr">
+        <is>
+          <t>완료</t>
         </is>
       </c>
     </row>
@@ -1902,7 +1988,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E65"/>
+  <dimension ref="A1:E74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2947,12 +3033,12 @@
       </c>
       <c r="B44" s="13" t="inlineStr">
         <is>
-          <t>직원 명단 관리</t>
+          <t>운영 인프라 안정화 (WS1~WS10)</t>
         </is>
       </c>
       <c r="C44" s="12" t="inlineStr">
         <is>
-          <t>직원</t>
+          <t>인프라</t>
         </is>
       </c>
       <c r="D44" s="14" t="inlineStr">
@@ -2960,7 +3046,11 @@
           <t>✅ 완료</t>
         </is>
       </c>
-      <c r="E44" s="13" t="inlineStr"/>
+      <c r="E44" s="13" t="inlineStr">
+        <is>
+          <t>Docker·보안·로깅·예외·헬스/관측</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="12" t="n">
@@ -2968,12 +3058,12 @@
       </c>
       <c r="B45" s="13" t="inlineStr">
         <is>
-          <t>부서별 담당 색상 배지 표시</t>
+          <t>입출고 내역 2·3차 정비 (main 머지)</t>
         </is>
       </c>
       <c r="C45" s="12" t="inlineStr">
         <is>
-          <t>직원</t>
+          <t>입출고</t>
         </is>
       </c>
       <c r="D45" s="14" t="inlineStr">
@@ -2981,7 +3071,11 @@
           <t>✅ 완료</t>
         </is>
       </c>
-      <c r="E45" s="13" t="inlineStr"/>
+      <c r="E45" s="13" t="inlineStr">
+        <is>
+          <t>model·process_step·department 파라미터</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="12" t="n">
@@ -2989,12 +3083,12 @@
       </c>
       <c r="B46" s="13" t="inlineStr">
         <is>
-          <t>작업자 PIN 로그인 + 감사 이력</t>
+          <t>모바일 UI/UX 전면 개편</t>
         </is>
       </c>
       <c r="C46" s="12" t="inlineStr">
         <is>
-          <t>보안</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="D46" s="14" t="inlineStr">
@@ -3004,7 +3098,7 @@
       </c>
       <c r="E46" s="13" t="inlineStr">
         <is>
-          <t>수정 이력 자동 기록</t>
+          <t>5개 화면 반응형 + 디자이너 PASS</t>
         </is>
       </c>
     </row>
@@ -3014,12 +3108,12 @@
       </c>
       <c r="B47" s="13" t="inlineStr">
         <is>
-          <t>로그인 및 권한 관리</t>
+          <t>불량 처리 흐름 재설계 Phase 1</t>
         </is>
       </c>
       <c r="C47" s="12" t="inlineStr">
         <is>
-          <t>보안</t>
+          <t>생산</t>
         </is>
       </c>
       <c r="D47" s="14" t="inlineStr">
@@ -3029,7 +3123,7 @@
       </c>
       <c r="E47" s="13" t="inlineStr">
         <is>
-          <t>PIN 기반 — 역할별 접근 제어 예정</t>
+          <t>라인 결재·격리·처리·테스트 113건</t>
         </is>
       </c>
     </row>
@@ -3039,12 +3133,12 @@
       </c>
       <c r="B48" s="13" t="inlineStr">
         <is>
-          <t>PC 화면 (데스크톱)</t>
+          <t>BOM 워크벤치 3-column + 완료 워크플로</t>
         </is>
       </c>
       <c r="C48" s="12" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>BOM</t>
         </is>
       </c>
       <c r="D48" s="14" t="inlineStr">
@@ -3052,7 +3146,11 @@
           <t>✅ 완료</t>
         </is>
       </c>
-      <c r="E48" s="13" t="inlineStr"/>
+      <c r="E48" s="13" t="inlineStr">
+        <is>
+          <t>BOM 완료 상태 토글 + export</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="12" t="n">
@@ -3060,12 +3158,12 @@
       </c>
       <c r="B49" s="13" t="inlineStr">
         <is>
-          <t>모바일 화면</t>
+          <t>입출고 CSV 외부 감시 시스템</t>
         </is>
       </c>
       <c r="C49" s="12" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>인프라</t>
         </is>
       </c>
       <c r="D49" s="14" t="inlineStr">
@@ -3073,7 +3171,11 @@
           <t>✅ 완료</t>
         </is>
       </c>
-      <c r="E49" s="13" t="inlineStr"/>
+      <c r="E49" s="13" t="inlineStr">
+        <is>
+          <t>월별 누적 미러</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="12" t="n">
@@ -3081,12 +3183,12 @@
       </c>
       <c r="B50" s="13" t="inlineStr">
         <is>
-          <t>다크 / 라이트 모드</t>
+          <t>ItemCode 도메인 정리</t>
         </is>
       </c>
       <c r="C50" s="12" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>인프라</t>
         </is>
       </c>
       <c r="D50" s="14" t="inlineStr">
@@ -3094,7 +3196,11 @@
           <t>✅ 완료</t>
         </is>
       </c>
-      <c r="E50" s="13" t="inlineStr"/>
+      <c r="E50" s="13" t="inlineStr">
+        <is>
+          <t>erp_code 잔재 정리</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="12" t="n">
@@ -3102,12 +3208,12 @@
       </c>
       <c r="B51" s="13" t="inlineStr">
         <is>
-          <t>관리자 화면</t>
+          <t>외부 PC 첫 실행 안정화</t>
         </is>
       </c>
       <c r="C51" s="12" t="inlineStr">
         <is>
-          <t>관리</t>
+          <t>인프라</t>
         </is>
       </c>
       <c r="D51" s="14" t="inlineStr">
@@ -3115,7 +3221,11 @@
           <t>✅ 완료</t>
         </is>
       </c>
-      <c r="E51" s="13" t="inlineStr"/>
+      <c r="E51" s="13" t="inlineStr">
+        <is>
+          <t>gitattributes + start.bat 사전 검사</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="12" t="n">
@@ -3123,12 +3233,12 @@
       </c>
       <c r="B52" s="13" t="inlineStr">
         <is>
-          <t>부서 관리 (DnD · 컬러 피커 · 검색)</t>
+          <t>권동환 5월 재고 100% 검증</t>
         </is>
       </c>
       <c r="C52" s="12" t="inlineStr">
         <is>
-          <t>관리</t>
+          <t>데이터</t>
         </is>
       </c>
       <c r="D52" s="14" t="inlineStr">
@@ -3136,7 +3246,11 @@
           <t>✅ 완료</t>
         </is>
       </c>
-      <c r="E52" s="13" t="inlineStr"/>
+      <c r="E52" s="13" t="inlineStr">
+        <is>
+          <t>엑셀↔DB 동기화·자식 행 반영</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="12" t="n">
@@ -3144,12 +3258,12 @@
       </c>
       <c r="B53" s="13" t="inlineStr">
         <is>
-          <t>데이터 CSV 내보내기</t>
+          <t>직원 명단 관리</t>
         </is>
       </c>
       <c r="C53" s="12" t="inlineStr">
         <is>
-          <t>관리</t>
+          <t>직원</t>
         </is>
       </c>
       <c r="D53" s="14" t="inlineStr">
@@ -3165,12 +3279,12 @@
       </c>
       <c r="B54" s="13" t="inlineStr">
         <is>
-          <t>원클릭 실행 (start.bat)</t>
+          <t>부서별 담당 색상 배지 표시</t>
         </is>
       </c>
       <c r="C54" s="12" t="inlineStr">
         <is>
-          <t>인프라</t>
+          <t>직원</t>
         </is>
       </c>
       <c r="D54" s="14" t="inlineStr">
@@ -3186,12 +3300,12 @@
       </c>
       <c r="B55" s="13" t="inlineStr">
         <is>
-          <t>테스트 자동화 (CI)</t>
+          <t>작업자 PIN 로그인 + 감사 이력</t>
         </is>
       </c>
       <c r="C55" s="12" t="inlineStr">
         <is>
-          <t>인프라</t>
+          <t>보안</t>
         </is>
       </c>
       <c r="D55" s="14" t="inlineStr">
@@ -3201,7 +3315,7 @@
       </c>
       <c r="E55" s="13" t="inlineStr">
         <is>
-          <t>pytest 42건 + vitest 12건</t>
+          <t>수정 이력 자동 기록</t>
         </is>
       </c>
     </row>
@@ -3211,237 +3325,434 @@
       </c>
       <c r="B56" s="13" t="inlineStr">
         <is>
+          <t>로그인 및 권한 관리</t>
+        </is>
+      </c>
+      <c r="C56" s="12" t="inlineStr">
+        <is>
+          <t>보안</t>
+        </is>
+      </c>
+      <c r="D56" s="14" t="inlineStr">
+        <is>
+          <t>✅ 완료</t>
+        </is>
+      </c>
+      <c r="E56" s="13" t="inlineStr">
+        <is>
+          <t>PIN 기반 — 역할별 접근 제어 예정</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="12" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="13" t="inlineStr">
+        <is>
+          <t>PC 화면 (데스크톱)</t>
+        </is>
+      </c>
+      <c r="C57" s="12" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="D57" s="14" t="inlineStr">
+        <is>
+          <t>✅ 완료</t>
+        </is>
+      </c>
+      <c r="E57" s="13" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="12" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" s="13" t="inlineStr">
+        <is>
+          <t>모바일 화면</t>
+        </is>
+      </c>
+      <c r="C58" s="12" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="D58" s="14" t="inlineStr">
+        <is>
+          <t>✅ 완료</t>
+        </is>
+      </c>
+      <c r="E58" s="13" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="12" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="13" t="inlineStr">
+        <is>
+          <t>다크 / 라이트 모드</t>
+        </is>
+      </c>
+      <c r="C59" s="12" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="D59" s="14" t="inlineStr">
+        <is>
+          <t>✅ 완료</t>
+        </is>
+      </c>
+      <c r="E59" s="13" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="12" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" s="13" t="inlineStr">
+        <is>
+          <t>관리자 화면</t>
+        </is>
+      </c>
+      <c r="C60" s="12" t="inlineStr">
+        <is>
+          <t>관리</t>
+        </is>
+      </c>
+      <c r="D60" s="14" t="inlineStr">
+        <is>
+          <t>✅ 완료</t>
+        </is>
+      </c>
+      <c r="E60" s="13" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="12" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" s="13" t="inlineStr">
+        <is>
+          <t>부서 관리 (DnD · 컬러 피커 · 검색)</t>
+        </is>
+      </c>
+      <c r="C61" s="12" t="inlineStr">
+        <is>
+          <t>관리</t>
+        </is>
+      </c>
+      <c r="D61" s="14" t="inlineStr">
+        <is>
+          <t>✅ 완료</t>
+        </is>
+      </c>
+      <c r="E61" s="13" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="12" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" s="13" t="inlineStr">
+        <is>
+          <t>데이터 CSV 내보내기</t>
+        </is>
+      </c>
+      <c r="C62" s="12" t="inlineStr">
+        <is>
+          <t>관리</t>
+        </is>
+      </c>
+      <c r="D62" s="14" t="inlineStr">
+        <is>
+          <t>✅ 완료</t>
+        </is>
+      </c>
+      <c r="E62" s="13" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="12" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" s="13" t="inlineStr">
+        <is>
+          <t>원클릭 실행 (start.bat)</t>
+        </is>
+      </c>
+      <c r="C63" s="12" t="inlineStr">
+        <is>
+          <t>인프라</t>
+        </is>
+      </c>
+      <c r="D63" s="14" t="inlineStr">
+        <is>
+          <t>✅ 완료</t>
+        </is>
+      </c>
+      <c r="E63" s="13" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="12" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" s="13" t="inlineStr">
+        <is>
+          <t>테스트 자동화 (CI)</t>
+        </is>
+      </c>
+      <c r="C64" s="12" t="inlineStr">
+        <is>
+          <t>인프라</t>
+        </is>
+      </c>
+      <c r="D64" s="14" t="inlineStr">
+        <is>
+          <t>✅ 완료</t>
+        </is>
+      </c>
+      <c r="E64" s="13" t="inlineStr">
+        <is>
+          <t>pytest 42건 + vitest 12건</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="12" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" s="13" t="inlineStr">
+        <is>
           <t>WAL-safe 백업 / 복구</t>
         </is>
       </c>
-      <c r="C56" s="12" t="inlineStr">
+      <c r="C65" s="12" t="inlineStr">
         <is>
           <t>인프라</t>
         </is>
       </c>
-      <c r="D56" s="14" t="inlineStr">
+      <c r="D65" s="14" t="inlineStr">
         <is>
           <t>✅ 완료</t>
         </is>
       </c>
-      <c r="E56" s="13" t="inlineStr">
+      <c r="E65" s="13" t="inlineStr">
         <is>
           <t>ops 스크립트 자동화</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="15" t="n">
-        <v>56</v>
-      </c>
-      <c r="B57" s="16" t="inlineStr">
-        <is>
-          <t>입출고 화면·내역 흐름 재설계</t>
-        </is>
-      </c>
-      <c r="C57" s="15" t="inlineStr">
-        <is>
-          <t>입출고</t>
-        </is>
-      </c>
-      <c r="D57" s="17" t="inlineStr">
+    <row r="66">
+      <c r="A66" s="15" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" s="16" t="inlineStr">
+        <is>
+          <t>실 재고 데이터 입력 + 직원 테스트</t>
+        </is>
+      </c>
+      <c r="C66" s="15" t="inlineStr">
+        <is>
+          <t>데이터</t>
+        </is>
+      </c>
+      <c r="D66" s="17" t="inlineStr">
         <is>
           <t>🔲 예정</t>
         </is>
       </c>
-      <c r="E57" s="16" t="inlineStr">
-        <is>
-          <t>담당자 동선 분석 후 (다음 주~다다음주)</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="15" t="n">
-        <v>57</v>
-      </c>
-      <c r="B58" s="16" t="inlineStr">
-        <is>
-          <t>실 재고 데이터 입력 + 직원 테스트</t>
-        </is>
-      </c>
-      <c r="C58" s="15" t="inlineStr">
-        <is>
-          <t>데이터</t>
-        </is>
-      </c>
-      <c r="D58" s="17" t="inlineStr">
+      <c r="E66" s="16" t="inlineStr">
+        <is>
+          <t>BOM·입출고 정리 후</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="15" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" s="16" t="inlineStr">
+        <is>
+          <t>불량 처리 흐름 Phase 2</t>
+        </is>
+      </c>
+      <c r="C67" s="15" t="inlineStr">
+        <is>
+          <t>생산</t>
+        </is>
+      </c>
+      <c r="D67" s="17" t="inlineStr">
         <is>
           <t>🔲 예정</t>
         </is>
       </c>
-      <c r="E58" s="16" t="inlineStr">
-        <is>
-          <t>BOM·입출고 정리 후</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="15" t="n">
-        <v>58</v>
-      </c>
-      <c r="B59" s="16" t="inlineStr">
+      <c r="E67" s="16" t="inlineStr">
+        <is>
+          <t>부서 결재·집계·자동화</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="15" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" s="16" t="inlineStr">
         <is>
           <t>역할별 접근 권한 연동</t>
         </is>
       </c>
-      <c r="C59" s="15" t="inlineStr">
+      <c r="C68" s="15" t="inlineStr">
         <is>
           <t>보안</t>
         </is>
       </c>
-      <c r="D59" s="17" t="inlineStr">
+      <c r="D68" s="17" t="inlineStr">
         <is>
           <t>🔲 예정</t>
         </is>
       </c>
-      <c r="E59" s="16" t="inlineStr">
+      <c r="E68" s="16" t="inlineStr">
         <is>
           <t>부서·역할 기반 (PIN 로그인 완료)</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="15" t="n">
-        <v>59</v>
-      </c>
-      <c r="B60" s="16" t="inlineStr">
+    <row r="69">
+      <c r="A69" s="15" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" s="16" t="inlineStr">
         <is>
           <t>총재고 / 가용재고 / 예약재고 분리</t>
         </is>
       </c>
-      <c r="C60" s="15" t="inlineStr">
+      <c r="C69" s="15" t="inlineStr">
         <is>
           <t>재고</t>
         </is>
       </c>
-      <c r="D60" s="17" t="inlineStr">
+      <c r="D69" s="17" t="inlineStr">
         <is>
           <t>🔲 예정</t>
         </is>
       </c>
-      <c r="E60" s="16" t="inlineStr">
+      <c r="E69" s="16" t="inlineStr">
         <is>
           <t>재고 가용성 계산 고도화</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="15" t="n">
-        <v>60</v>
-      </c>
-      <c r="B61" s="16" t="inlineStr">
+    <row r="70">
+      <c r="A70" s="15" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" s="16" t="inlineStr">
         <is>
           <t>외부 접근 환경 구성</t>
         </is>
       </c>
-      <c r="C61" s="15" t="inlineStr">
+      <c r="C70" s="15" t="inlineStr">
         <is>
           <t>인프라</t>
         </is>
       </c>
-      <c r="D61" s="17" t="inlineStr">
+      <c r="D70" s="17" t="inlineStr">
         <is>
           <t>🔲 예정</t>
         </is>
       </c>
-      <c r="E61" s="16" t="inlineStr">
+      <c r="E70" s="16" t="inlineStr">
         <is>
           <t>PC 또는 NAS 서버 + API 인증</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="15" t="n">
-        <v>61</v>
-      </c>
-      <c r="B62" s="16" t="inlineStr">
+    <row r="71">
+      <c r="A71" s="15" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" s="16" t="inlineStr">
         <is>
           <t>발주 관리</t>
         </is>
       </c>
-      <c r="C62" s="15" t="inlineStr">
+      <c r="C71" s="15" t="inlineStr">
         <is>
           <t>구매</t>
         </is>
       </c>
-      <c r="D62" s="17" t="inlineStr">
+      <c r="D71" s="17" t="inlineStr">
         <is>
           <t>🔲 예정</t>
         </is>
       </c>
-      <c r="E62" s="16" t="inlineStr"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="15" t="n">
-        <v>62</v>
-      </c>
-      <c r="B63" s="16" t="inlineStr">
+      <c r="E71" s="16" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="15" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" s="16" t="inlineStr">
         <is>
           <t>생산 실적 / 원가 관리</t>
         </is>
       </c>
-      <c r="C63" s="15" t="inlineStr">
+      <c r="C72" s="15" t="inlineStr">
         <is>
           <t>생산</t>
         </is>
       </c>
-      <c r="D63" s="17" t="inlineStr">
+      <c r="D72" s="17" t="inlineStr">
         <is>
           <t>🔲 예정</t>
         </is>
       </c>
-      <c r="E63" s="16" t="inlineStr"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="15" t="n">
-        <v>63</v>
-      </c>
-      <c r="B64" s="16" t="inlineStr">
+      <c r="E72" s="16" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="15" t="n">
+        <v>72</v>
+      </c>
+      <c r="B73" s="16" t="inlineStr">
         <is>
           <t>부서별 생산진행도 대시보드</t>
         </is>
       </c>
-      <c r="C64" s="15" t="inlineStr">
+      <c r="C73" s="15" t="inlineStr">
         <is>
           <t>관리</t>
         </is>
       </c>
-      <c r="D64" s="17" t="inlineStr">
+      <c r="D73" s="17" t="inlineStr">
         <is>
           <t>🔲 예정</t>
         </is>
       </c>
-      <c r="E64" s="16" t="inlineStr">
+      <c r="E73" s="16" t="inlineStr">
         <is>
           <t>사장님 요청 — 검토 중</t>
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="15" t="n">
-        <v>64</v>
-      </c>
-      <c r="B65" s="16" t="inlineStr">
+    <row r="74">
+      <c r="A74" s="15" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" s="16" t="inlineStr">
         <is>
           <t>출하 거래처 관리</t>
         </is>
       </c>
-      <c r="C65" s="15" t="inlineStr">
+      <c r="C74" s="15" t="inlineStr">
         <is>
           <t>출하</t>
         </is>
       </c>
-      <c r="D65" s="17" t="inlineStr">
+      <c r="D74" s="17" t="inlineStr">
         <is>
           <t>🔲 예정</t>
         </is>
       </c>
-      <c r="E65" s="16" t="inlineStr">
+      <c r="E74" s="16" t="inlineStr">
         <is>
           <t>거래처 마스터 + 출하 이력</t>
         </is>
@@ -3458,7 +3769,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4183,7 +4494,7 @@
         </is>
       </c>
       <c r="B31" s="9" t="n">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="C31" s="10" t="inlineStr">
         <is>
@@ -4195,6 +4506,50 @@
         </is>
       </c>
       <c r="D31" s="9" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="50" customHeight="1">
+      <c r="A32" s="18" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B32" s="18" t="n">
+        <v>11</v>
+      </c>
+      <c r="C32" s="19" t="inlineStr">
+        <is>
+          <t>2026-05-21 docs: 자체 MES 구축 PR — 1:1 보고용 슬라이드 데크(pr.html)
+2026-05-21 data: 권동환 5월 재고 매칭 - 폴더 정리·사용자 수작업 파일·후보 보조표 스크립트
+2026-05-21 data: 5월 입출고 audit 로그 갱신 — SR-20260520-052533 불량처
+2026-05-21 docs: PR 슬라이드 톤 다듬기 + 환율 정정 ($1=1,500원)
+chore: ERP/erp → MES 표기 일괄 정리 — 도메인 erp_code 식별자는 보존</t>
+        </is>
+      </c>
+      <c r="D32" s="18" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="50" customHeight="1">
+      <c r="A33" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B33" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C33" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-22 chore: vault-sync 코드 작업 일괄 반영 (vault/ 제외, 85파일)</t>
+        </is>
+      </c>
+      <c r="D33" s="9" t="inlineStr">
         <is>
           <t>Frontend</t>
         </is>
@@ -4211,7 +4566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F537"/>
+  <dimension ref="A1:F571"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -21406,6 +21761,1094 @@
         </is>
       </c>
     </row>
+    <row r="538">
+      <c r="A538" s="18" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B538" s="18" t="inlineStr">
+        <is>
+          <t>08:55</t>
+        </is>
+      </c>
+      <c r="C538" s="18" t="inlineStr">
+        <is>
+          <t>a5b858aa</t>
+        </is>
+      </c>
+      <c r="D538" s="19" t="inlineStr">
+        <is>
+          <t>2026-05-20 admin: 외부 심사용 입출고 CSV 미러 시스템 (자동 누적 + 월별 다운로드)</t>
+        </is>
+      </c>
+      <c r="E538" s="18" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="F538" s="18" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B539" s="9" t="inlineStr">
+        <is>
+          <t>08:56</t>
+        </is>
+      </c>
+      <c r="C539" s="9" t="inlineStr">
+        <is>
+          <t>91231f96</t>
+        </is>
+      </c>
+      <c r="D539" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-20 docs: 개발현황 엑셀에 근무 외 작업 시각화 추가</t>
+        </is>
+      </c>
+      <c r="E539" s="9" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="F539" s="9" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" s="18" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B540" s="18" t="inlineStr">
+        <is>
+          <t>09:01</t>
+        </is>
+      </c>
+      <c r="C540" s="18" t="inlineStr">
+        <is>
+          <t>ddae2e2c</t>
+        </is>
+      </c>
+      <c r="D540" s="19" t="inlineStr">
+        <is>
+          <t>2026-05-20 admin: OpenAPI baseline 재생성 (audit-csv 라우터 4종 반영)</t>
+        </is>
+      </c>
+      <c r="E540" s="18" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="F540" s="18" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B541" s="9" t="inlineStr">
+        <is>
+          <t>09:24</t>
+        </is>
+      </c>
+      <c r="C541" s="9" t="inlineStr">
+        <is>
+          <t>14943b3f</t>
+        </is>
+      </c>
+      <c r="D541" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-20 desktop: 입출고 내역 알약 정합 (BOM ± 부호, 구분·단건 통일 폭, 일시/구분 중앙정렬)</t>
+        </is>
+      </c>
+      <c r="E541" s="9" t="inlineStr">
+        <is>
+          <t>desktop</t>
+        </is>
+      </c>
+      <c r="F541" s="9" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" s="18" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B542" s="18" t="inlineStr">
+        <is>
+          <t>09:47</t>
+        </is>
+      </c>
+      <c r="C542" s="18" t="inlineStr">
+        <is>
+          <t>e91f1fe1</t>
+        </is>
+      </c>
+      <c r="D542" s="19" t="inlineStr">
+        <is>
+          <t>2026-05-20 backend: 주간보고 모델 매트릭스 ProductSymbol DB 기반 동적 매핑</t>
+        </is>
+      </c>
+      <c r="E542" s="18" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F542" s="18" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B543" s="9" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="C543" s="9" t="inlineStr">
+        <is>
+          <t>4db421a2</t>
+        </is>
+      </c>
+      <c r="D543" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-20 backend: F4b 완료 — UtcDatetime을 전체 응답 스키마로 확산 (9h 오차 근본 수정)</t>
+        </is>
+      </c>
+      <c r="E543" s="9" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F543" s="9" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" s="18" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B544" s="18" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="C544" s="18" t="inlineStr">
+        <is>
+          <t>ab38bcf0</t>
+        </is>
+      </c>
+      <c r="D544" s="19" t="inlineStr">
+        <is>
+          <t>2026-05-20 docs: F4b 완료에 따라 작업 계획 문서 제거</t>
+        </is>
+      </c>
+      <c r="E544" s="18" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="F544" s="18" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B545" s="9" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="C545" s="9" t="inlineStr">
+        <is>
+          <t>5ce4e17a</t>
+        </is>
+      </c>
+      <c r="D545" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-20 desktop: 대시보드 필터 버튼을 생산가능 행 우측으로 이동</t>
+        </is>
+      </c>
+      <c r="E545" s="9" t="inlineStr">
+        <is>
+          <t>desktop</t>
+        </is>
+      </c>
+      <c r="F545" s="9" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" s="18" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B546" s="18" t="inlineStr">
+        <is>
+          <t>10:36</t>
+        </is>
+      </c>
+      <c r="C546" s="18" t="inlineStr">
+        <is>
+          <t>e8ddce86</t>
+        </is>
+      </c>
+      <c r="D546" s="19" t="inlineStr">
+        <is>
+          <t>2026-05-20 backend: OpenAPI baseline 갱신 — EmployeeResponse format:date-time 복원</t>
+        </is>
+      </c>
+      <c r="E546" s="18" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F546" s="18" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B547" s="9" t="inlineStr">
+        <is>
+          <t>10:40</t>
+        </is>
+      </c>
+      <c r="C547" s="9" t="inlineStr">
+        <is>
+          <t>bff4a081</t>
+        </is>
+      </c>
+      <c r="D547" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-20 desktop: 입출고 내역 좌측 잔손 — ADJUST 묶음 수량·메모 셀·자동 접힘·담당자 정리</t>
+        </is>
+      </c>
+      <c r="E547" s="9" t="inlineStr">
+        <is>
+          <t>desktop</t>
+        </is>
+      </c>
+      <c r="F547" s="9" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" s="18" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B548" s="18" t="inlineStr">
+        <is>
+          <t>10:42</t>
+        </is>
+      </c>
+      <c r="C548" s="18" t="inlineStr">
+        <is>
+          <t>6730961c</t>
+        </is>
+      </c>
+      <c r="D548" s="19" t="inlineStr">
+        <is>
+          <t>2026-05-20 desktop: 주간보고 공정별 변화 카드 픽셀 조정 + 5월 입출고 감사 CSV</t>
+        </is>
+      </c>
+      <c r="E548" s="18" t="inlineStr">
+        <is>
+          <t>desktop</t>
+        </is>
+      </c>
+      <c r="F548" s="18" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B549" s="9" t="inlineStr">
+        <is>
+          <t>11:03</t>
+        </is>
+      </c>
+      <c r="C549" s="9" t="inlineStr">
+        <is>
+          <t>7f735504</t>
+        </is>
+      </c>
+      <c r="D549" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-20 refactor: queue/alerts/counts dead 기능 흔적 제거 + CLAUDE.md 갱신</t>
+        </is>
+      </c>
+      <c r="E549" s="9" t="inlineStr">
+        <is>
+          <t>refactor</t>
+        </is>
+      </c>
+      <c r="F549" s="9" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" s="18" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B550" s="18" t="inlineStr">
+        <is>
+          <t>11:04</t>
+        </is>
+      </c>
+      <c r="C550" s="18" t="inlineStr">
+        <is>
+          <t>cab3e4f1</t>
+        </is>
+      </c>
+      <c r="D550" s="19" t="inlineStr">
+        <is>
+          <t>Merge feat/cleanup-dead-pages: queue/alerts/counts dead 기능 흔적 제거</t>
+        </is>
+      </c>
+      <c r="E550" s="18" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="F550" s="18" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B551" s="9" t="inlineStr">
+        <is>
+          <t>11:58</t>
+        </is>
+      </c>
+      <c r="C551" s="9" t="inlineStr">
+        <is>
+          <t>7c7edeb7</t>
+        </is>
+      </c>
+      <c r="D551" s="10" t="inlineStr">
+        <is>
+          <t>chore: separate dev baselines from attic</t>
+        </is>
+      </c>
+      <c r="E551" s="9" t="inlineStr">
+        <is>
+          <t>chore</t>
+        </is>
+      </c>
+      <c r="F551" s="9" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" s="18" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B552" s="18" t="inlineStr">
+        <is>
+          <t>12:44</t>
+        </is>
+      </c>
+      <c r="C552" s="18" t="inlineStr">
+        <is>
+          <t>f1695796</t>
+        </is>
+      </c>
+      <c r="D552" s="19" t="inlineStr">
+        <is>
+          <t>2026-05-20 desktop: 입출고 내역 우측 카드 재정비 — Hero 통합·좌측 톤 일관</t>
+        </is>
+      </c>
+      <c r="E552" s="18" t="inlineStr">
+        <is>
+          <t>desktop</t>
+        </is>
+      </c>
+      <c r="F552" s="18" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B553" s="9" t="inlineStr">
+        <is>
+          <t>12:44</t>
+        </is>
+      </c>
+      <c r="C553" s="9" t="inlineStr">
+        <is>
+          <t>50979139</t>
+        </is>
+      </c>
+      <c r="D553" s="10" t="inlineStr">
+        <is>
+          <t>Merge feat/history-phase4: 입출고 내역 우측 카드 재정비</t>
+        </is>
+      </c>
+      <c r="E553" s="9" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="F553" s="9" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" s="18" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B554" s="18" t="inlineStr">
+        <is>
+          <t>13:33</t>
+        </is>
+      </c>
+      <c r="C554" s="18" t="inlineStr">
+        <is>
+          <t>f22065dc</t>
+        </is>
+      </c>
+      <c r="D554" s="19" t="inlineStr">
+        <is>
+          <t>2026-05-20 desktop: BOM/단품 chip 도 구분 열 FlowBadge 규칙으로 통일 (min-w-6.5rem · px-3 py-1 · text-xs · tracking-wide)</t>
+        </is>
+      </c>
+      <c r="E554" s="18" t="inlineStr">
+        <is>
+          <t>desktop</t>
+        </is>
+      </c>
+      <c r="F554" s="18" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B555" s="9" t="inlineStr">
+        <is>
+          <t>13:34</t>
+        </is>
+      </c>
+      <c r="C555" s="9" t="inlineStr">
+        <is>
+          <t>e3a7c033</t>
+        </is>
+      </c>
+      <c r="D555" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-20 desktop: BOM 워크벤치 잘린 품목명·코드 호버 시 풀네임 툴팁</t>
+        </is>
+      </c>
+      <c r="E555" s="9" t="inlineStr">
+        <is>
+          <t>desktop</t>
+        </is>
+      </c>
+      <c r="F555" s="9" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" s="18" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B556" s="18" t="inlineStr">
+        <is>
+          <t>16:52</t>
+        </is>
+      </c>
+      <c r="C556" s="18" t="inlineStr">
+        <is>
+          <t>77c5df46</t>
+        </is>
+      </c>
+      <c r="D556" s="19" t="inlineStr">
+        <is>
+          <t>2026-05-20 docs: 발표 대본 초안 SCRIPT.md 추가</t>
+        </is>
+      </c>
+      <c r="E556" s="18" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="F556" s="18" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B557" s="9" t="inlineStr">
+        <is>
+          <t>16:52</t>
+        </is>
+      </c>
+      <c r="C557" s="9" t="inlineStr">
+        <is>
+          <t>db7ae55d</t>
+        </is>
+      </c>
+      <c r="D557" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-20 desktop: 부서 내 작업 흐름 표시 — batch.from==to 면 그 부서 단일 표기</t>
+        </is>
+      </c>
+      <c r="E557" s="9" t="inlineStr">
+        <is>
+          <t>desktop</t>
+        </is>
+      </c>
+      <c r="F557" s="9" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" s="18" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B558" s="18" t="inlineStr">
+        <is>
+          <t>16:53</t>
+        </is>
+      </c>
+      <c r="C558" s="18" t="inlineStr">
+        <is>
+          <t>188582d4</t>
+        </is>
+      </c>
+      <c r="D558" s="19" t="inlineStr">
+        <is>
+          <t>2026-05-20 backend: 품목 추가 시 erp_code 시리얼 카테고리 전역 스코프 + sort_order 자동 부여</t>
+        </is>
+      </c>
+      <c r="E558" s="18" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F558" s="18" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B559" s="9" t="inlineStr">
+        <is>
+          <t>16:56</t>
+        </is>
+      </c>
+      <c r="C559" s="9" t="inlineStr">
+        <is>
+          <t>ebf71d31</t>
+        </is>
+      </c>
+      <c r="D559" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-20 data: 권동환 5월 재고 ↔ MES 마스터 매칭 산출물·스크립트</t>
+        </is>
+      </c>
+      <c r="E559" s="9" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="F559" s="9" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" s="18" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B560" s="18" t="inlineStr">
+        <is>
+          <t>11:53</t>
+        </is>
+      </c>
+      <c r="C560" s="18" t="inlineStr">
+        <is>
+          <t>cb178b8d</t>
+        </is>
+      </c>
+      <c r="D560" s="19" t="inlineStr">
+        <is>
+          <t>2026-05-21 docs: 자체 MES 구축 PR — 1:1 보고용 슬라이드 데크(pr.html)</t>
+        </is>
+      </c>
+      <c r="E560" s="18" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="F560" s="18" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B561" s="9" t="inlineStr">
+        <is>
+          <t>11:56</t>
+        </is>
+      </c>
+      <c r="C561" s="9" t="inlineStr">
+        <is>
+          <t>a246db65</t>
+        </is>
+      </c>
+      <c r="D561" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-21 data: 권동환 5월 재고 매칭 - 폴더 정리·사용자 수작업 파일·후보 보조표 스크립트</t>
+        </is>
+      </c>
+      <c r="E561" s="9" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="F561" s="9" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" s="18" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B562" s="18" t="inlineStr">
+        <is>
+          <t>12:01</t>
+        </is>
+      </c>
+      <c r="C562" s="18" t="inlineStr">
+        <is>
+          <t>21e98cdf</t>
+        </is>
+      </c>
+      <c r="D562" s="19" t="inlineStr">
+        <is>
+          <t>2026-05-21 data: 5월 입출고 audit 로그 갱신 — SR-20260520-052533 불량처리 승인 기록 1건</t>
+        </is>
+      </c>
+      <c r="E562" s="18" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="F562" s="18" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B563" s="9" t="inlineStr">
+        <is>
+          <t>12:57</t>
+        </is>
+      </c>
+      <c r="C563" s="9" t="inlineStr">
+        <is>
+          <t>00feb4c7</t>
+        </is>
+      </c>
+      <c r="D563" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-21 docs: PR 슬라이드 톤 다듬기 + 환율 정정 ($1=1,500원)</t>
+        </is>
+      </c>
+      <c r="E563" s="9" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="F563" s="9" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" s="18" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B564" s="18" t="inlineStr">
+        <is>
+          <t>14:17</t>
+        </is>
+      </c>
+      <c r="C564" s="18" t="inlineStr">
+        <is>
+          <t>214020e1</t>
+        </is>
+      </c>
+      <c r="D564" s="19" t="inlineStr">
+        <is>
+          <t>chore: ERP/erp → MES 표기 일괄 정리 — 도메인 erp_code 식별자는 보존</t>
+        </is>
+      </c>
+      <c r="E564" s="18" t="inlineStr">
+        <is>
+          <t>chore</t>
+        </is>
+      </c>
+      <c r="F564" s="18" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B565" s="9" t="inlineStr">
+        <is>
+          <t>14:26</t>
+        </is>
+      </c>
+      <c r="C565" s="9" t="inlineStr">
+        <is>
+          <t>b792f7a0</t>
+        </is>
+      </c>
+      <c r="D565" s="10" t="inlineStr">
+        <is>
+          <t>refactor: 입출고 내역 구분 라벨 — 죽은 거래 타입 5종 완전 제거</t>
+        </is>
+      </c>
+      <c r="E565" s="9" t="inlineStr">
+        <is>
+          <t>refactor</t>
+        </is>
+      </c>
+      <c r="F565" s="9" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" s="18" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B566" s="18" t="inlineStr">
+        <is>
+          <t>14:36</t>
+        </is>
+      </c>
+      <c r="C566" s="18" t="inlineStr">
+        <is>
+          <t>33b9e321</t>
+        </is>
+      </c>
+      <c r="D566" s="19" t="inlineStr">
+        <is>
+          <t>docs: 발표 슬라이드 파일명 변경 — 교육.html / 비교.html</t>
+        </is>
+      </c>
+      <c r="E566" s="18" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="F566" s="18" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B567" s="9" t="inlineStr">
+        <is>
+          <t>15:54</t>
+        </is>
+      </c>
+      <c r="C567" s="9" t="inlineStr">
+        <is>
+          <t>f1ff96ce</t>
+        </is>
+      </c>
+      <c r="D567" s="10" t="inlineStr">
+        <is>
+          <t>chore: items.item_code 통합 + ErpCode → ItemCode 도메인 rename</t>
+        </is>
+      </c>
+      <c r="E567" s="9" t="inlineStr">
+        <is>
+          <t>chore</t>
+        </is>
+      </c>
+      <c r="F567" s="9" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" s="18" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B568" s="18" t="inlineStr">
+        <is>
+          <t>15:58</t>
+        </is>
+      </c>
+      <c r="C568" s="18" t="inlineStr">
+        <is>
+          <t>4d5861a6</t>
+        </is>
+      </c>
+      <c r="D568" s="19" t="inlineStr">
+        <is>
+          <t>docs: 불량 처리 흐름 재설계 문서 추가</t>
+        </is>
+      </c>
+      <c r="E568" s="18" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="F568" s="18" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B569" s="9" t="inlineStr">
+        <is>
+          <t>16:33</t>
+        </is>
+      </c>
+      <c r="C569" s="9" t="inlineStr">
+        <is>
+          <t>c6aa0eb8</t>
+        </is>
+      </c>
+      <c r="D569" s="10" t="inlineStr">
+        <is>
+          <t>chore: ERP 잔재 후속 정리 — cosmetic + 누락된 진짜 잔재</t>
+        </is>
+      </c>
+      <c r="E569" s="9" t="inlineStr">
+        <is>
+          <t>chore</t>
+        </is>
+      </c>
+      <c r="F569" s="9" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" s="18" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B570" s="18" t="inlineStr">
+        <is>
+          <t>16:39</t>
+        </is>
+      </c>
+      <c r="C570" s="18" t="inlineStr">
+        <is>
+          <t>fe1c1ba1</t>
+        </is>
+      </c>
+      <c r="D570" s="19" t="inlineStr">
+        <is>
+          <t>chore: 외부 PC 첫 실행 안정화 — .gitattributes + start.bat 사전 검사</t>
+        </is>
+      </c>
+      <c r="E570" s="18" t="inlineStr">
+        <is>
+          <t>chore</t>
+        </is>
+      </c>
+      <c r="F570" s="18" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B571" s="9" t="inlineStr">
+        <is>
+          <t>16:32</t>
+        </is>
+      </c>
+      <c r="C571" s="9" t="inlineStr">
+        <is>
+          <t>174ba759</t>
+        </is>
+      </c>
+      <c r="D571" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-22 chore: vault-sync 코드 작업 일괄 반영 (vault/ 제외, 85파일)</t>
+        </is>
+      </c>
+      <c r="E571" s="9" t="inlineStr">
+        <is>
+          <t>chore</t>
+        </is>
+      </c>
+      <c r="F571" s="9" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
2026-06-08 docs: 주간보고 6/1~6/5 갱신 + 자동화 스킬 추가
## 주간보고 갱신
- 6/1~6/5 진행 사항 11개 항목 추가 (코드정비, 인수인계 기능 추가 등)
- 도입부 톤 수정 ("이번 주" → "저번 주")
- txt/xlsx 동기화

## update-weekly-report 스킬 생성
- ~/.claude/skills/update-weekly-report/ 구성
- SKILL.md: 스킬 설명 및 사용 가이드
- README.md: 상세 사용 방법
- scripts/update_weekly_report.py: 자동화 스크립트
  * 날짜/도입부/항목 대화형 입력
  * md/txt/xlsx 3개 파일 한 번에 자동 갱신

## 메모리 추가
- feedback_weekly_report_tone.md: 권동환 사원님 피드백 (톤 개선 규칙)
- MEMORY.md 인덱스 업데이트

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_attic/docs/개발현황.xlsx
+++ b/_attic/docs/개발현황.xlsx
@@ -570,7 +570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E52"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="67.25" customWidth="1" min="1" max="1"/>
@@ -616,7 +616,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>831건 (회사 기간 670건)</t>
+          <t>876건 (회사 기간 670건)</t>
         </is>
       </c>
     </row>
@@ -628,7 +628,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>304건 (평일 야간·주말·휴가 시간 커밋)</t>
+          <t>325건 (평일 야간·주말·휴가 시간 커밋)</t>
         </is>
       </c>
     </row>
@@ -1869,20 +1869,61 @@
               <color rgb="00000000"/>
               <sz val="10"/>
             </rPr>
-            <t>■■■■■■■■</t>
+            <t>■■■■■■■■■■</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00ED7D31"/>
+              <sz val="10"/>
+            </rPr>
+            <t>■■■■</t>
           </r>
           <r>
             <rPr>
               <color rgb="00000000"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">  (16)</t>
+            <t xml:space="preserve">  (29)</t>
           </r>
         </is>
       </c>
     </row>
+    <row r="53" ht="18" customHeight="1">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">2026-06-05  </t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+              <sz val="10"/>
+            </rPr>
+            <t>■■■■■■■■■■</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00ED7D31"/>
+              <sz val="10"/>
+            </rPr>
+            <t>■■■■■■</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">  (32)</t>
+          </r>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="50">
+  <mergeCells count="51">
     <mergeCell ref="A30:E30"/>
     <mergeCell ref="A39:E39"/>
     <mergeCell ref="A34:E34"/>
@@ -1919,6 +1960,7 @@
     <mergeCell ref="A14:E14"/>
     <mergeCell ref="A22:E22"/>
     <mergeCell ref="A17:E17"/>
+    <mergeCell ref="A53:E53"/>
     <mergeCell ref="A29:E29"/>
     <mergeCell ref="A35:E35"/>
     <mergeCell ref="B8:E8"/>
@@ -4369,7 +4411,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D43"/>
+  <dimension ref="A1:D44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5377,7 +5419,7 @@
         </is>
       </c>
       <c r="B43" s="7" t="n">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="C43" s="8" t="inlineStr">
         <is>
@@ -5390,7 +5432,31 @@
       </c>
       <c r="D43" s="7" t="inlineStr">
         <is>
-          <t>Frontend</t>
+          <t>Backend</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="67.5" customHeight="1">
+      <c r="A44" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B44" s="15" t="n">
+        <v>32</v>
+      </c>
+      <c r="C44" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-05 frontend: 인수인계 UX 개선 + 인수인계 도착 알림
+2026-06-05 docs: 피드백 현황 갱신 — F1~F5 구현 반영 (해결 5건)
+2026-06-05 chore: gitignore .understand-anything 산출물
+2026-06-05 backend: schemas.py → schemas/ 도메인별 패키지 분리
+2026-06-05 docs: legacy/_warehouse_v2 폴더 오해 방지 README 추가</t>
+        </is>
+      </c>
+      <c r="D44" s="15" t="inlineStr">
+        <is>
+          <t>Backend</t>
         </is>
       </c>
     </row>
@@ -5405,7 +5471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F832"/>
+  <dimension ref="A1:F877"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -32040,6 +32106,1446 @@
         </is>
       </c>
     </row>
+    <row r="833">
+      <c r="A833" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B833" s="7" t="inlineStr">
+        <is>
+          <t>16:25</t>
+        </is>
+      </c>
+      <c r="C833" s="7" t="inlineStr">
+        <is>
+          <t>1bea7ea7</t>
+        </is>
+      </c>
+      <c r="D833" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-04 docs: 이지훈 피드백 2건 추가 + 직원연락망·인수인계 자료 보관</t>
+        </is>
+      </c>
+      <c r="E833" s="7" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="F833" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B834" s="15" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="C834" s="15" t="inlineStr">
+        <is>
+          <t>4a3e549b</t>
+        </is>
+      </c>
+      <c r="D834" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-04 docs: 주간보고 5/30~6/4 최종 — 호칭 정정 + 사용자 수정분 반영</t>
+        </is>
+      </c>
+      <c r="E834" s="15" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="F834" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="835">
+      <c r="A835" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B835" s="7" t="inlineStr">
+        <is>
+          <t>16:56</t>
+        </is>
+      </c>
+      <c r="C835" s="7" t="inlineStr">
+        <is>
+          <t>2abe513a</t>
+        </is>
+      </c>
+      <c r="D835" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-04 frontend: 창고 지도 — 브라우저 뒤로가기·박스 hover·줄 구분·다중 품목코드</t>
+        </is>
+      </c>
+      <c r="E835" s="7" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F835" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" s="19" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B836" s="19" t="inlineStr">
+        <is>
+          <t>17:09</t>
+        </is>
+      </c>
+      <c r="C836" s="19" t="inlineStr">
+        <is>
+          <t>ff0c1f2e</t>
+        </is>
+      </c>
+      <c r="D836" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-04 io: 입출고 임시저장 덮어쓰기 제거 — batch_id 분기로 새 슬롯 누적</t>
+        </is>
+      </c>
+      <c r="E836" s="19" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="F836" s="21" t="inlineStr">
+        <is>
+          <t>근무 외</t>
+        </is>
+      </c>
+    </row>
+    <row r="837">
+      <c r="A837" s="19" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B837" s="19" t="inlineStr">
+        <is>
+          <t>17:16</t>
+        </is>
+      </c>
+      <c r="C837" s="19" t="inlineStr">
+        <is>
+          <t>cd621bc3</t>
+        </is>
+      </c>
+      <c r="D837" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-04 defect: 재작업 분해 시 회수 외 자식 → 격리 이동 (소실 차단)</t>
+        </is>
+      </c>
+      <c r="E837" s="19" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="F837" s="21" t="inlineStr">
+        <is>
+          <t>근무 외</t>
+        </is>
+      </c>
+    </row>
+    <row r="838">
+      <c r="A838" s="19" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B838" s="19" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="C838" s="19" t="inlineStr">
+        <is>
+          <t>494fb287</t>
+        </is>
+      </c>
+      <c r="D838" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-04 notify: 결재 알림 시스템 — 요청 도착/승인/반려 (F2·F3)</t>
+        </is>
+      </c>
+      <c r="E838" s="19" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="F838" s="21" t="inlineStr">
+        <is>
+          <t>근무 외</t>
+        </is>
+      </c>
+    </row>
+    <row r="839">
+      <c r="A839" s="19" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B839" s="19" t="inlineStr">
+        <is>
+          <t>17:52</t>
+        </is>
+      </c>
+      <c r="C839" s="19" t="inlineStr">
+        <is>
+          <t>03cd6fb3</t>
+        </is>
+      </c>
+      <c r="D839" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-04 handover: 튜브→고압/진공 인수인계서 (작성·인수확인·자동이동·인쇄) (F1)</t>
+        </is>
+      </c>
+      <c r="E839" s="19" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="F839" s="21" t="inlineStr">
+        <is>
+          <t>근무 외</t>
+        </is>
+      </c>
+    </row>
+    <row r="840">
+      <c r="A840" s="19" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B840" s="19" t="inlineStr">
+        <is>
+          <t>17:54</t>
+        </is>
+      </c>
+      <c r="C840" s="19" t="inlineStr">
+        <is>
+          <t>5ab1634f</t>
+        </is>
+      </c>
+      <c r="D840" s="20" t="inlineStr">
+        <is>
+          <t>Merge feat/io-draft-stacking (F5): 입출고 임시저장 누적</t>
+        </is>
+      </c>
+      <c r="E840" s="19" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="F840" s="21" t="inlineStr">
+        <is>
+          <t>근무 외</t>
+        </is>
+      </c>
+    </row>
+    <row r="841">
+      <c r="A841" s="19" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B841" s="19" t="inlineStr">
+        <is>
+          <t>17:54</t>
+        </is>
+      </c>
+      <c r="C841" s="19" t="inlineStr">
+        <is>
+          <t>d9a360cb</t>
+        </is>
+      </c>
+      <c r="D841" s="20" t="inlineStr">
+        <is>
+          <t>Merge feat/rework-quarantine (F4): 재작업 회수 외 자식 격리 이동</t>
+        </is>
+      </c>
+      <c r="E841" s="19" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="F841" s="21" t="inlineStr">
+        <is>
+          <t>근무 외</t>
+        </is>
+      </c>
+    </row>
+    <row r="842">
+      <c r="A842" s="19" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B842" s="19" t="inlineStr">
+        <is>
+          <t>17:54</t>
+        </is>
+      </c>
+      <c r="C842" s="19" t="inlineStr">
+        <is>
+          <t>3130c356</t>
+        </is>
+      </c>
+      <c r="D842" s="20" t="inlineStr">
+        <is>
+          <t>Merge feat/approval-notifications (F2·F3): 결재 알림 시스템</t>
+        </is>
+      </c>
+      <c r="E842" s="19" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="F842" s="21" t="inlineStr">
+        <is>
+          <t>근무 외</t>
+        </is>
+      </c>
+    </row>
+    <row r="843">
+      <c r="A843" s="19" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B843" s="19" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="C843" s="19" t="inlineStr">
+        <is>
+          <t>0f1fcb1b</t>
+        </is>
+      </c>
+      <c r="D843" s="20" t="inlineStr">
+        <is>
+          <t>Merge feat/handover-doc (F1): 튜브→고압/진공 인수인계서</t>
+        </is>
+      </c>
+      <c r="E843" s="19" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="F843" s="21" t="inlineStr">
+        <is>
+          <t>근무 외</t>
+        </is>
+      </c>
+    </row>
+    <row r="844">
+      <c r="A844" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B844" s="15" t="inlineStr">
+        <is>
+          <t>16:56</t>
+        </is>
+      </c>
+      <c r="C844" s="15" t="inlineStr">
+        <is>
+          <t>6302eeec</t>
+        </is>
+      </c>
+      <c r="D844" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-04 frontend: 창고 지도 — 브라우저 뒤로가기·박스 hover·줄 구분·다중 품목코드</t>
+        </is>
+      </c>
+      <c r="E844" s="15" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F844" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="845">
+      <c r="A845" s="19" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B845" s="19" t="inlineStr">
+        <is>
+          <t>19:40</t>
+        </is>
+      </c>
+      <c r="C845" s="19" t="inlineStr">
+        <is>
+          <t>796578de</t>
+        </is>
+      </c>
+      <c r="D845" s="20" t="inlineStr">
+        <is>
+          <t>Merge pull request #21 from Hw-03/docs/feedback-handover-2026-06-04</t>
+        </is>
+      </c>
+      <c r="E845" s="19" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="F845" s="21" t="inlineStr">
+        <is>
+          <t>근무 외</t>
+        </is>
+      </c>
+    </row>
+    <row r="846">
+      <c r="A846" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B846" s="15" t="inlineStr">
+        <is>
+          <t>09:04</t>
+        </is>
+      </c>
+      <c r="C846" s="15" t="inlineStr">
+        <is>
+          <t>9ab9e66a</t>
+        </is>
+      </c>
+      <c r="D846" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-05 frontend: 인수인계 UX 개선 + 인수인계 도착 알림</t>
+        </is>
+      </c>
+      <c r="E846" s="15" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F846" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="847">
+      <c r="A847" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B847" s="7" t="inlineStr">
+        <is>
+          <t>09:38</t>
+        </is>
+      </c>
+      <c r="C847" s="7" t="inlineStr">
+        <is>
+          <t>51db7f8e</t>
+        </is>
+      </c>
+      <c r="D847" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-05 docs: 피드백 현황 갱신 — F1~F5 구현 반영 (해결 5건)</t>
+        </is>
+      </c>
+      <c r="E847" s="7" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="F847" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="848">
+      <c r="A848" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B848" s="15" t="inlineStr">
+        <is>
+          <t>10:29</t>
+        </is>
+      </c>
+      <c r="C848" s="15" t="inlineStr">
+        <is>
+          <t>3bba6cbf</t>
+        </is>
+      </c>
+      <c r="D848" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-05 chore: gitignore .understand-anything 산출물</t>
+        </is>
+      </c>
+      <c r="E848" s="15" t="inlineStr">
+        <is>
+          <t>chore</t>
+        </is>
+      </c>
+      <c r="F848" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="849">
+      <c r="A849" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B849" s="7" t="inlineStr">
+        <is>
+          <t>11:57</t>
+        </is>
+      </c>
+      <c r="C849" s="7" t="inlineStr">
+        <is>
+          <t>4333ee7d</t>
+        </is>
+      </c>
+      <c r="D849" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-05 backend: schemas.py → schemas/ 도메인별 패키지 분리</t>
+        </is>
+      </c>
+      <c r="E849" s="7" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F849" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="850">
+      <c r="A850" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B850" s="15" t="inlineStr">
+        <is>
+          <t>11:57</t>
+        </is>
+      </c>
+      <c r="C850" s="15" t="inlineStr">
+        <is>
+          <t>6ffbdf6e</t>
+        </is>
+      </c>
+      <c r="D850" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-05 docs: legacy/_warehouse_v2 폴더 오해 방지 README 추가</t>
+        </is>
+      </c>
+      <c r="E850" s="15" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="F850" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="851">
+      <c r="A851" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B851" s="7" t="inlineStr">
+        <is>
+          <t>11:57</t>
+        </is>
+      </c>
+      <c r="C851" s="7" t="inlineStr">
+        <is>
+          <t>59f656f4</t>
+        </is>
+      </c>
+      <c r="D851" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-05 backend: transactions.py 필터/응답 헬퍼 → _tx_filters.py 분리</t>
+        </is>
+      </c>
+      <c r="E851" s="7" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F851" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="852">
+      <c r="A852" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B852" s="15" t="inlineStr">
+        <is>
+          <t>12:27</t>
+        </is>
+      </c>
+      <c r="C852" s="15" t="inlineStr">
+        <is>
+          <t>b7e3b330</t>
+        </is>
+      </c>
+      <c r="D852" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-05 frontend: 인수인계 인쇄 — 로고 base64 임베드 + A4 문서 레이아웃</t>
+        </is>
+      </c>
+      <c r="E852" s="15" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F852" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="853">
+      <c r="A853" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B853" s="7" t="inlineStr">
+        <is>
+          <t>13:35</t>
+        </is>
+      </c>
+      <c r="C853" s="7" t="inlineStr">
+        <is>
+          <t>5f36fa1a</t>
+        </is>
+      </c>
+      <c r="D853" s="8" t="inlineStr">
+        <is>
+          <t>Merge remote-tracking branch 'origin/refactor/cleancode-review-prep'</t>
+        </is>
+      </c>
+      <c r="E853" s="7" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="F853" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="854">
+      <c r="A854" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B854" s="15" t="inlineStr">
+        <is>
+          <t>13:35</t>
+        </is>
+      </c>
+      <c r="C854" s="15" t="inlineStr">
+        <is>
+          <t>a9388922</t>
+        </is>
+      </c>
+      <c r="D854" s="16" t="inlineStr">
+        <is>
+          <t>Merge remote-tracking branch 'origin/docs/feedback-f1f5-resolved'</t>
+        </is>
+      </c>
+      <c r="E854" s="15" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="F854" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="855">
+      <c r="A855" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B855" s="7" t="inlineStr">
+        <is>
+          <t>13:35</t>
+        </is>
+      </c>
+      <c r="C855" s="7" t="inlineStr">
+        <is>
+          <t>34ac5d93</t>
+        </is>
+      </c>
+      <c r="D855" s="8" t="inlineStr">
+        <is>
+          <t>Merge remote-tracking branch 'origin/feat/handover-print-template'</t>
+        </is>
+      </c>
+      <c r="E855" s="7" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="F855" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="856">
+      <c r="A856" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B856" s="15" t="inlineStr">
+        <is>
+          <t>14:03</t>
+        </is>
+      </c>
+      <c r="C856" s="15" t="inlineStr">
+        <is>
+          <t>d16218f3</t>
+        </is>
+      </c>
+      <c r="D856" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-05 data: 튜브-고압 인수인계서 보관 (pdf·docx)</t>
+        </is>
+      </c>
+      <c r="E856" s="15" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="F856" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="857">
+      <c r="A857" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B857" s="7" t="inlineStr">
+        <is>
+          <t>14:07</t>
+        </is>
+      </c>
+      <c r="C857" s="7" t="inlineStr">
+        <is>
+          <t>5b1058a9</t>
+        </is>
+      </c>
+      <c r="D857" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-05 chore: 완료 플랜 _attic/docs/research 보관 (cleancode-review-prep)</t>
+        </is>
+      </c>
+      <c r="E857" s="7" t="inlineStr">
+        <is>
+          <t>chore</t>
+        </is>
+      </c>
+      <c r="F857" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="858">
+      <c r="A858" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B858" s="15" t="inlineStr">
+        <is>
+          <t>14:18</t>
+        </is>
+      </c>
+      <c r="C858" s="15" t="inlineStr">
+        <is>
+          <t>7b3f968e</t>
+        </is>
+      </c>
+      <c r="D858" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-05 frontend: Pretendard 폰트 self-host 로드</t>
+        </is>
+      </c>
+      <c r="E858" s="15" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F858" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="859">
+      <c r="A859" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B859" s="7" t="inlineStr">
+        <is>
+          <t>14:22</t>
+        </is>
+      </c>
+      <c r="C859" s="7" t="inlineStr">
+        <is>
+          <t>e37cf2d9</t>
+        </is>
+      </c>
+      <c r="D859" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-05 docs: 모바일 디자인 시스템 문서 실측 정정</t>
+        </is>
+      </c>
+      <c r="E859" s="7" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="F859" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="860">
+      <c r="A860" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B860" s="15" t="inlineStr">
+        <is>
+          <t>14:33</t>
+        </is>
+      </c>
+      <c r="C860" s="15" t="inlineStr">
+        <is>
+          <t>5b85a2ba</t>
+        </is>
+      </c>
+      <c r="D860" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-05 refactor: 모바일 중복 primitive 정리 — 죽은 EmptyState 제거·분리 명시</t>
+        </is>
+      </c>
+      <c r="E860" s="15" t="inlineStr">
+        <is>
+          <t>refactor</t>
+        </is>
+      </c>
+      <c r="F860" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="861">
+      <c r="A861" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B861" s="7" t="inlineStr">
+        <is>
+          <t>14:40</t>
+        </is>
+      </c>
+      <c r="C861" s="7" t="inlineStr">
+        <is>
+          <t>3a4becc3</t>
+        </is>
+      </c>
+      <c r="D861" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-05 frontend: features/mes 디자인 규칙 ESLint 가드 추가</t>
+        </is>
+      </c>
+      <c r="E861" s="7" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F861" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="862">
+      <c r="A862" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B862" s="15" t="inlineStr">
+        <is>
+          <t>14:47</t>
+        </is>
+      </c>
+      <c r="C862" s="15" t="inlineStr">
+        <is>
+          <t>7eae9897</t>
+        </is>
+      </c>
+      <c r="D862" s="16" t="inlineStr">
+        <is>
+          <t>Merge branch 'feat/design-consistency'</t>
+        </is>
+      </c>
+      <c r="E862" s="15" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="F862" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="863">
+      <c r="A863" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B863" s="7" t="inlineStr">
+        <is>
+          <t>15:34</t>
+        </is>
+      </c>
+      <c r="C863" s="7" t="inlineStr">
+        <is>
+          <t>0cadee07</t>
+        </is>
+      </c>
+      <c r="D863" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-05 frontend: 불량 탭 디자인 정합 — 표준 primitive·토큰으로 통일</t>
+        </is>
+      </c>
+      <c r="E863" s="7" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F863" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="864">
+      <c r="A864" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B864" s="15" t="inlineStr">
+        <is>
+          <t>16:31</t>
+        </is>
+      </c>
+      <c r="C864" s="15" t="inlineStr">
+        <is>
+          <t>95f6a989</t>
+        </is>
+      </c>
+      <c r="D864" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-05 frontend: 불량 탭 3장 카드 진입 화면 + 바로 폐기 전 품목화</t>
+        </is>
+      </c>
+      <c r="E864" s="15" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F864" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="865">
+      <c r="A865" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B865" s="7" t="inlineStr">
+        <is>
+          <t>16:54</t>
+        </is>
+      </c>
+      <c r="C865" s="7" t="inlineStr">
+        <is>
+          <t>328e313e</t>
+        </is>
+      </c>
+      <c r="D865" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-05 docs: 이계숙 주임 피드백 2건 등록 (구두)</t>
+        </is>
+      </c>
+      <c r="E865" s="7" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="F865" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="866">
+      <c r="A866" s="19" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B866" s="19" t="inlineStr">
+        <is>
+          <t>18:24</t>
+        </is>
+      </c>
+      <c r="C866" s="19" t="inlineStr">
+        <is>
+          <t>b577189a</t>
+        </is>
+      </c>
+      <c r="D866" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-05 frontend: 미사용 features/mes 빈 골조 7파일 제거</t>
+        </is>
+      </c>
+      <c r="E866" s="19" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F866" s="21" t="inlineStr">
+        <is>
+          <t>근무 외</t>
+        </is>
+      </c>
+    </row>
+    <row r="867">
+      <c r="A867" s="19" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B867" s="19" t="inlineStr">
+        <is>
+          <t>18:24</t>
+        </is>
+      </c>
+      <c r="C867" s="19" t="inlineStr">
+        <is>
+          <t>1c402557</t>
+        </is>
+      </c>
+      <c r="D867" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-05 frontend: 죽은 _archive 컴포넌트 4파일 제거 (import 깨짐·미사용)</t>
+        </is>
+      </c>
+      <c r="E867" s="19" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F867" s="21" t="inlineStr">
+        <is>
+          <t>근무 외</t>
+        </is>
+      </c>
+    </row>
+    <row r="868">
+      <c r="A868" s="19" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B868" s="19" t="inlineStr">
+        <is>
+          <t>18:24</t>
+        </is>
+      </c>
+      <c r="C868" s="19" t="inlineStr">
+        <is>
+          <t>e61e12c4</t>
+        </is>
+      </c>
+      <c r="D868" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-05 frontend: features/mes 전용 ESLint overrides 블록 제거</t>
+        </is>
+      </c>
+      <c r="E868" s="19" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F868" s="21" t="inlineStr">
+        <is>
+          <t>근무 외</t>
+        </is>
+      </c>
+    </row>
+    <row r="869">
+      <c r="A869" s="19" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B869" s="19" t="inlineStr">
+        <is>
+          <t>18:25</t>
+        </is>
+      </c>
+      <c r="C869" s="19" t="inlineStr">
+        <is>
+          <t>6e7a637e</t>
+        </is>
+      </c>
+      <c r="D869" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-05 frontend: app/legacy → app/mes 개명 + 앱 라우트 /legacy→/mes</t>
+        </is>
+      </c>
+      <c r="E869" s="19" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F869" s="21" t="inlineStr">
+        <is>
+          <t>근무 외</t>
+        </is>
+      </c>
+    </row>
+    <row r="870">
+      <c r="A870" s="19" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B870" s="19" t="inlineStr">
+        <is>
+          <t>18:25</t>
+        </is>
+      </c>
+      <c r="C870" s="19" t="inlineStr">
+        <is>
+          <t>bbd7ed0f</t>
+        </is>
+      </c>
+      <c r="D870" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-05 frontend: e2e·모바일 스크립트 라우트 /legacy→/mes 갱신</t>
+        </is>
+      </c>
+      <c r="E870" s="19" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F870" s="21" t="inlineStr">
+        <is>
+          <t>근무 외</t>
+        </is>
+      </c>
+    </row>
+    <row r="871">
+      <c r="A871" s="19" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B871" s="19" t="inlineStr">
+        <is>
+          <t>18:35</t>
+        </is>
+      </c>
+      <c r="C871" s="19" t="inlineStr">
+        <is>
+          <t>a4a74eaa</t>
+        </is>
+      </c>
+      <c r="D871" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-05 fix: app/legacy→mes 개명 누락 참조 수정 (drift 테스트 경로·docstring·CLAUDE.md·README)</t>
+        </is>
+      </c>
+      <c r="E871" s="19" t="inlineStr">
+        <is>
+          <t>fix</t>
+        </is>
+      </c>
+      <c r="F871" s="21" t="inlineStr">
+        <is>
+          <t>근무 외</t>
+        </is>
+      </c>
+    </row>
+    <row r="872">
+      <c r="A872" s="19" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B872" s="19" t="inlineStr">
+        <is>
+          <t>18:46</t>
+        </is>
+      </c>
+      <c r="C872" s="19" t="inlineStr">
+        <is>
+          <t>a7a99eb4</t>
+        </is>
+      </c>
+      <c r="D872" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-05 frontend: e2e io-defect 로케이터 수정 — filter 방식으로 공백 의존성 제거</t>
+        </is>
+      </c>
+      <c r="E872" s="19" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F872" s="21" t="inlineStr">
+        <is>
+          <t>근무 외</t>
+        </is>
+      </c>
+    </row>
+    <row r="873">
+      <c r="A873" s="19" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B873" s="19" t="inlineStr">
+        <is>
+          <t>18:46</t>
+        </is>
+      </c>
+      <c r="C873" s="19" t="inlineStr">
+        <is>
+          <t>0dfff902</t>
+        </is>
+      </c>
+      <c r="D873" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-05 frontend: e2e io-defect 로케이터 수정 — filter 방식으로 공백 의존성 제거</t>
+        </is>
+      </c>
+      <c r="E873" s="19" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F873" s="21" t="inlineStr">
+        <is>
+          <t>근무 외</t>
+        </is>
+      </c>
+    </row>
+    <row r="874">
+      <c r="A874" s="19" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B874" s="19" t="inlineStr">
+        <is>
+          <t>18:52</t>
+        </is>
+      </c>
+      <c r="C874" s="19" t="inlineStr">
+        <is>
+          <t>e0a29b5d</t>
+        </is>
+      </c>
+      <c r="D874" s="20" t="inlineStr">
+        <is>
+          <t>Merge remote-tracking branch 'origin/main' into refactor/legacy-to-mes</t>
+        </is>
+      </c>
+      <c r="E874" s="19" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="F874" s="21" t="inlineStr">
+        <is>
+          <t>근무 외</t>
+        </is>
+      </c>
+    </row>
+    <row r="875">
+      <c r="A875" s="19" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B875" s="19" t="inlineStr">
+        <is>
+          <t>19:05</t>
+        </is>
+      </c>
+      <c r="C875" s="19" t="inlineStr">
+        <is>
+          <t>04d4ab17</t>
+        </is>
+      </c>
+      <c r="D875" s="20" t="inlineStr">
+        <is>
+          <t>Merge branch 'refactor/legacy-to-mes' into HEAD</t>
+        </is>
+      </c>
+      <c r="E875" s="19" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="F875" s="21" t="inlineStr">
+        <is>
+          <t>근무 외</t>
+        </is>
+      </c>
+    </row>
+    <row r="876">
+      <c r="A876" s="19" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B876" s="19" t="inlineStr">
+        <is>
+          <t>19:06</t>
+        </is>
+      </c>
+      <c r="C876" s="19" t="inlineStr">
+        <is>
+          <t>7f7815f5</t>
+        </is>
+      </c>
+      <c r="D876" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-05 docs: legacy→mes 개명 완료 플랜 _attic/docs/research 보관</t>
+        </is>
+      </c>
+      <c r="E876" s="19" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="F876" s="21" t="inlineStr">
+        <is>
+          <t>근무 외</t>
+        </is>
+      </c>
+    </row>
+    <row r="877">
+      <c r="A877" s="19" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B877" s="19" t="inlineStr">
+        <is>
+          <t>23:08</t>
+        </is>
+      </c>
+      <c r="C877" s="19" t="inlineStr">
+        <is>
+          <t>e5a612b9</t>
+        </is>
+      </c>
+      <c r="D877" s="20" t="inlineStr">
+        <is>
+          <t>Merge branch 'docs/feedback-lee-gye-suk-2026-06-05'</t>
+        </is>
+      </c>
+      <c r="E877" s="19" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="F877" s="21" t="inlineStr">
+        <is>
+          <t>근무 외</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
2026-06-10 docs: 주간보고 6/8~6/10 갱신
</commit_message>
<xml_diff>
--- a/_attic/docs/개발현황.xlsx
+++ b/_attic/docs/개발현황.xlsx
@@ -570,7 +570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="67.25" customWidth="1" min="1" max="1"/>
@@ -616,7 +616,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>876건 (회사 기간 670건)</t>
+          <t>920건 (회사 기간 670건)</t>
         </is>
       </c>
     </row>
@@ -628,7 +628,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>325건 (평일 야간·주말·휴가 시간 커밋)</t>
+          <t>326건 (평일 야간·주말·휴가 시간 커밋)</t>
         </is>
       </c>
     </row>
@@ -1922,8 +1922,89 @@
         </is>
       </c>
     </row>
+    <row r="54" ht="18" customHeight="1">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">2026-06-08  </t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+              <sz val="10"/>
+            </rPr>
+            <t>■■■■■■■■■■■■■■■</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">  (31)</t>
+          </r>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="18" customHeight="1">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">2026-06-09  </t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+              <sz val="10"/>
+            </rPr>
+            <t>■■■■</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">  (9)</t>
+          </r>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="18" customHeight="1">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">2026-06-10  </t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+              <sz val="10"/>
+            </rPr>
+            <t>■■</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">  (4)</t>
+          </r>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="51">
+  <mergeCells count="54">
     <mergeCell ref="A30:E30"/>
     <mergeCell ref="A39:E39"/>
     <mergeCell ref="A34:E34"/>
@@ -1940,6 +2021,7 @@
     <mergeCell ref="A36:E36"/>
     <mergeCell ref="B4:E4"/>
     <mergeCell ref="A16:E16"/>
+    <mergeCell ref="A54:E54"/>
     <mergeCell ref="A25:E25"/>
     <mergeCell ref="A41:E41"/>
     <mergeCell ref="B7:E7"/>
@@ -1948,7 +2030,9 @@
     <mergeCell ref="A46:E46"/>
     <mergeCell ref="A18:E18"/>
     <mergeCell ref="A27:E27"/>
+    <mergeCell ref="A56:E56"/>
     <mergeCell ref="A21:E21"/>
+    <mergeCell ref="A55:E55"/>
     <mergeCell ref="A12:E12"/>
     <mergeCell ref="A50:E50"/>
     <mergeCell ref="A26:E26"/>
@@ -4411,7 +4495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D44"/>
+  <dimension ref="A1:D47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5457,6 +5541,77 @@
       <c r="D44" s="15" t="inlineStr">
         <is>
           <t>Backend</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="67.5" customHeight="1">
+      <c r="A45" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B45" s="7" t="n">
+        <v>31</v>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-08 frontend: add useToggleSet hook (필터 토글 중복 통합용)
+2026-06-08 frontend: 필터 토글 12개를 useToggleSet 로 치환 (중복 제거)
+2026-06-08 chore: coverage 문서 임계 정정(50→75) + io_dispatch exc
+2026-06-08 frontend: 부서결재·draft React Query 훅 추가 (useDraftCa
+2026-06-08 frontend: 창고 패널 3종 손수 fetch→React Query 이관 (중복 제거</t>
+        </is>
+      </c>
+      <c r="D45" s="7" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="67.5" customHeight="1">
+      <c r="A46" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B46" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="C46" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-09 dev: add stop-frontend.ps1 + start.bat preflight 
+2026-06-09 frontend: 불량 탭 피드백 개선 — 부분 수량 복귀·부서 필터·KPI 카드 분리
+2026-06-09 frontend: 불량 탭 헤더 제거 + 뷰 전환 슬라이드 애니메이션
+2026-06-09 frontend: 창고 지도 UX 개선 (열 클릭·자리 분할·슬롯 번호)
+2026-06-09 defect: 불량 탭 UX 개선 (카트 흐름·뒤로가기·필터 정리)</t>
+        </is>
+      </c>
+      <c r="D46" s="15" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="54" customHeight="1">
+      <c r="A47" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B47" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-10 defect: 처리 패널 재설계 + 부서 접기/펼치기 UX
+2026-06-10 backend: unquarantine reason_category optional 처리
+2026-06-10 test: io-defect E2E 안정화 — 정상복귀 제출 셀렉터 모호성 해소
+2026-06-10 docs: 주간보고 6/7~6/10 갱신</t>
+        </is>
+      </c>
+      <c r="D47" s="7" t="inlineStr">
+        <is>
+          <t>Frontend</t>
         </is>
       </c>
     </row>
@@ -5471,7 +5626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F877"/>
+  <dimension ref="A1:F921"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -33546,6 +33701,1414 @@
         </is>
       </c>
     </row>
+    <row r="878">
+      <c r="A878" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B878" s="15" t="inlineStr">
+        <is>
+          <t>09:53</t>
+        </is>
+      </c>
+      <c r="C878" s="15" t="inlineStr">
+        <is>
+          <t>62ab44cb</t>
+        </is>
+      </c>
+      <c r="D878" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-08 frontend: add useToggleSet hook (필터 토글 중복 통합용)</t>
+        </is>
+      </c>
+      <c r="E878" s="15" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F878" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="879">
+      <c r="A879" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B879" s="7" t="inlineStr">
+        <is>
+          <t>09:53</t>
+        </is>
+      </c>
+      <c r="C879" s="7" t="inlineStr">
+        <is>
+          <t>17bd57e2</t>
+        </is>
+      </c>
+      <c r="D879" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-08 frontend: 필터 토글 12개를 useToggleSet 로 치환 (중복 제거)</t>
+        </is>
+      </c>
+      <c r="E879" s="7" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F879" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="880">
+      <c r="A880" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B880" s="15" t="inlineStr">
+        <is>
+          <t>11:06</t>
+        </is>
+      </c>
+      <c r="C880" s="15" t="inlineStr">
+        <is>
+          <t>c888a0d3</t>
+        </is>
+      </c>
+      <c r="D880" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-08 chore: coverage 문서 임계 정정(50→75) + io_dispatch except 의도 주석</t>
+        </is>
+      </c>
+      <c r="E880" s="15" t="inlineStr">
+        <is>
+          <t>chore</t>
+        </is>
+      </c>
+      <c r="F880" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="881">
+      <c r="A881" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B881" s="7" t="inlineStr">
+        <is>
+          <t>11:06</t>
+        </is>
+      </c>
+      <c r="C881" s="7" t="inlineStr">
+        <is>
+          <t>13218771</t>
+        </is>
+      </c>
+      <c r="D881" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-08 frontend: 부서결재·draft React Query 훅 추가 (useDraftCartQuery 신설)</t>
+        </is>
+      </c>
+      <c r="E881" s="7" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F881" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="882">
+      <c r="A882" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B882" s="15" t="inlineStr">
+        <is>
+          <t>11:06</t>
+        </is>
+      </c>
+      <c r="C882" s="15" t="inlineStr">
+        <is>
+          <t>70412baf</t>
+        </is>
+      </c>
+      <c r="D882" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-08 frontend: 창고 패널 3종 손수 fetch→React Query 이관 (중복 제거)</t>
+        </is>
+      </c>
+      <c r="E882" s="15" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F882" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="883">
+      <c r="A883" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B883" s="7" t="inlineStr">
+        <is>
+          <t>11:06</t>
+        </is>
+      </c>
+      <c r="C883" s="7" t="inlineStr">
+        <is>
+          <t>e656dd1c</t>
+        </is>
+      </c>
+      <c r="D883" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-08 frontend: AdminDepartmentsSection 하위 컴포넌트 분리 (큰 파일 정리)</t>
+        </is>
+      </c>
+      <c r="E883" s="7" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F883" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="884">
+      <c r="A884" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B884" s="15" t="inlineStr">
+        <is>
+          <t>11:06</t>
+        </is>
+      </c>
+      <c r="C884" s="15" t="inlineStr">
+        <is>
+          <t>f8b97196</t>
+        </is>
+      </c>
+      <c r="D884" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-08 frontend: AdminEmployeesSection 하위 컴포넌트 분리 (큰 파일 정리)</t>
+        </is>
+      </c>
+      <c r="E884" s="15" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F884" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="885">
+      <c r="A885" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B885" s="7" t="inlineStr">
+        <is>
+          <t>11:12</t>
+        </is>
+      </c>
+      <c r="C885" s="7" t="inlineStr">
+        <is>
+          <t>1e80dcda</t>
+        </is>
+      </c>
+      <c r="D885" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-08 docs: 주간보고 6/1~6/5 갱신 + 자동화 스킬 추가</t>
+        </is>
+      </c>
+      <c r="E885" s="7" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="F885" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="886">
+      <c r="A886" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B886" s="15" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="C886" s="15" t="inlineStr">
+        <is>
+          <t>366c584a</t>
+        </is>
+      </c>
+      <c r="D886" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-08 backend: EmployeeItemOrder 모델 추가 (직원별 품목 순서 저장 테이블)</t>
+        </is>
+      </c>
+      <c r="E886" s="15" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F886" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="887">
+      <c r="A887" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B887" s="7" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="C887" s="7" t="inlineStr">
+        <is>
+          <t>11617983</t>
+        </is>
+      </c>
+      <c r="D887" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-08 backend: MyItemOrder 스키마 추가 (개인 품목 순서 입출력)</t>
+        </is>
+      </c>
+      <c r="E887" s="7" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F887" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="888">
+      <c r="A888" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B888" s="15" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="C888" s="15" t="inlineStr">
+        <is>
+          <t>2e739bbf</t>
+        </is>
+      </c>
+      <c r="D888" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-08 backend: /api/items/my-order 라우터 추가 (GET/PUT/DELETE, 개인 순서·PIN 불필요)</t>
+        </is>
+      </c>
+      <c r="E888" s="15" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F888" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="889">
+      <c r="A889" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B889" s="7" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="C889" s="7" t="inlineStr">
+        <is>
+          <t>7c15195e</t>
+        </is>
+      </c>
+      <c r="D889" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-08 backend: my-order 엔드포인트 테스트 8건 추가</t>
+        </is>
+      </c>
+      <c r="E889" s="7" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F889" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="890">
+      <c r="A890" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B890" s="15" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="C890" s="15" t="inlineStr">
+        <is>
+          <t>e6e8eb8f</t>
+        </is>
+      </c>
+      <c r="D890" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-08 chore: OpenAPI baseline 갱신 (my-order 엔드포인트 반영)</t>
+        </is>
+      </c>
+      <c r="E890" s="15" t="inlineStr">
+        <is>
+          <t>chore</t>
+        </is>
+      </c>
+      <c r="F890" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="891">
+      <c r="A891" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B891" s="7" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="C891" s="7" t="inlineStr">
+        <is>
+          <t>bdca6aef</t>
+        </is>
+      </c>
+      <c r="D891" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-08 frontend: my-order API 함수·쿼리키 추가</t>
+        </is>
+      </c>
+      <c r="E891" s="7" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F891" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="892">
+      <c r="A892" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B892" s="15" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="C892" s="15" t="inlineStr">
+        <is>
+          <t>529dbfe4</t>
+        </is>
+      </c>
+      <c r="D892" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-08 frontend: useMyItemOrderQuery 훅 추가 (조회·저장·초기화)</t>
+        </is>
+      </c>
+      <c r="E892" s="15" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F892" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="893">
+      <c r="A893" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B893" s="7" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="C893" s="7" t="inlineStr">
+        <is>
+          <t>f20db273</t>
+        </is>
+      </c>
+      <c r="D893" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-08 frontend: useItemOrderDrag 드래그 훅 추가 (포인터 기반 재정렬)</t>
+        </is>
+      </c>
+      <c r="E893" s="7" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F893" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="894">
+      <c r="A894" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B894" s="15" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="C894" s="15" t="inlineStr">
+        <is>
+          <t>963cb4a8</t>
+        </is>
+      </c>
+      <c r="D894" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-08 frontend: buildEmployeeOrderRank 정렬 헬퍼 추가</t>
+        </is>
+      </c>
+      <c r="E894" s="15" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F894" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="895">
+      <c r="A895" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B895" s="7" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="C895" s="7" t="inlineStr">
+        <is>
+          <t>070bd67f</t>
+        </is>
+      </c>
+      <c r="D895" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-08 frontend: 입출고 품목창에 직원별 순서 정렬·편집 UI 적용</t>
+        </is>
+      </c>
+      <c r="E895" s="7" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F895" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="896">
+      <c r="A896" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B896" s="15" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="C896" s="15" t="inlineStr">
+        <is>
+          <t>7bb33fb5</t>
+        </is>
+      </c>
+      <c r="D896" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-08 frontend: 불량 품목창에 직원별 순서 정렬·편집 UI 적용 (테스트 QueryClient 주입)</t>
+        </is>
+      </c>
+      <c r="E896" s="15" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F896" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="897">
+      <c r="A897" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B897" s="7" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="C897" s="7" t="inlineStr">
+        <is>
+          <t>6733cc67</t>
+        </is>
+      </c>
+      <c r="D897" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-08 frontend: 격리 추가 검색결과에 직원별 순서 정렬 적용 (테스트 QueryClient 주입)</t>
+        </is>
+      </c>
+      <c r="E897" s="7" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F897" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="898">
+      <c r="A898" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B898" s="15" t="inlineStr">
+        <is>
+          <t>11:53</t>
+        </is>
+      </c>
+      <c r="C898" s="15" t="inlineStr">
+        <is>
+          <t>48f0c0b3</t>
+        </is>
+      </c>
+      <c r="D898" s="16" t="inlineStr">
+        <is>
+          <t>Merge pull request #29 from Hw-03/feat/employee-item-order</t>
+        </is>
+      </c>
+      <c r="E898" s="15" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="F898" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="899">
+      <c r="A899" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B899" s="7" t="inlineStr">
+        <is>
+          <t>12:54</t>
+        </is>
+      </c>
+      <c r="C899" s="7" t="inlineStr">
+        <is>
+          <t>98eca70d</t>
+        </is>
+      </c>
+      <c r="D899" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-08 backend: warehouse_map 라우터·서비스 테스트 신설</t>
+        </is>
+      </c>
+      <c r="E899" s="7" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F899" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="900">
+      <c r="A900" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B900" s="15" t="inlineStr">
+        <is>
+          <t>12:54</t>
+        </is>
+      </c>
+      <c r="C900" s="15" t="inlineStr">
+        <is>
+          <t>d285764b</t>
+        </is>
+      </c>
+      <c r="D900" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-08 backend: io_preview 라우팅·BOM 전개 단위 테스트 신설</t>
+        </is>
+      </c>
+      <c r="E900" s="15" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F900" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="901">
+      <c r="A901" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B901" s="7" t="inlineStr">
+        <is>
+          <t>12:54</t>
+        </is>
+      </c>
+      <c r="C901" s="7" t="inlineStr">
+        <is>
+          <t>9c039233</t>
+        </is>
+      </c>
+      <c r="D901" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-08 frontend: ItemDetailSheet fetch→React Query 이관 (+ useTransactionsQuery enabled 옵션)</t>
+        </is>
+      </c>
+      <c r="E901" s="7" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F901" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="902">
+      <c r="A902" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B902" s="15" t="inlineStr">
+        <is>
+          <t>13:59</t>
+        </is>
+      </c>
+      <c r="C902" s="15" t="inlineStr">
+        <is>
+          <t>63270d42</t>
+        </is>
+      </c>
+      <c r="D902" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-08 backend: io 제출 원자성 회귀 테스트 추가</t>
+        </is>
+      </c>
+      <c r="E902" s="15" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F902" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="903">
+      <c r="A903" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B903" s="7" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="C903" s="7" t="inlineStr">
+        <is>
+          <t>94508dd2</t>
+        </is>
+      </c>
+      <c r="D903" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-08 backend: Item·Inventory 조회 repository 도입·중복 통합</t>
+        </is>
+      </c>
+      <c r="E903" s="7" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F903" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="904">
+      <c r="A904" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B904" s="15" t="inlineStr">
+        <is>
+          <t>14:50</t>
+        </is>
+      </c>
+      <c r="C904" s="15" t="inlineStr">
+        <is>
+          <t>892c1701</t>
+        </is>
+      </c>
+      <c r="D904" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-08 docs: 허동현·이지훈 피드백 등록 (불량처리·창고지도·BOM)</t>
+        </is>
+      </c>
+      <c r="E904" s="15" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="F904" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="905">
+      <c r="A905" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B905" s="7" t="inlineStr">
+        <is>
+          <t>14:52</t>
+        </is>
+      </c>
+      <c r="C905" s="7" t="inlineStr">
+        <is>
+          <t>fde59b0d</t>
+        </is>
+      </c>
+      <c r="D905" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-08 docs: ERD 전면 현행화 — 25개 테이블 8개 도메인</t>
+        </is>
+      </c>
+      <c r="E905" s="7" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="F905" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="906">
+      <c r="A906" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B906" s="15" t="inlineStr">
+        <is>
+          <t>14:57</t>
+        </is>
+      </c>
+      <c r="C906" s="15" t="inlineStr">
+        <is>
+          <t>51760207</t>
+        </is>
+      </c>
+      <c r="D906" s="16" t="inlineStr">
+        <is>
+          <t>Merge pull request #30 from Hw-03/docs/feedback-huh-lee-20260608</t>
+        </is>
+      </c>
+      <c r="E906" s="15" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="F906" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="907">
+      <c r="A907" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B907" s="7" t="inlineStr">
+        <is>
+          <t>16:47</t>
+        </is>
+      </c>
+      <c r="C907" s="7" t="inlineStr">
+        <is>
+          <t>9f3d31b2</t>
+        </is>
+      </c>
+      <c r="D907" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-08 frontend: 창고 지도 위치 안내 UX 개선</t>
+        </is>
+      </c>
+      <c r="E907" s="7" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F907" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="908">
+      <c r="A908" s="19" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B908" s="19" t="inlineStr">
+        <is>
+          <t>19:23</t>
+        </is>
+      </c>
+      <c r="C908" s="19" t="inlineStr">
+        <is>
+          <t>5c83271f</t>
+        </is>
+      </c>
+      <c r="D908" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-08 backend: fix unhandled exception handler logging (exc_info=exc)</t>
+        </is>
+      </c>
+      <c r="E908" s="19" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F908" s="21" t="inlineStr">
+        <is>
+          <t>근무 외</t>
+        </is>
+      </c>
+    </row>
+    <row r="909">
+      <c r="A909" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B909" s="7" t="inlineStr">
+        <is>
+          <t>08:26</t>
+        </is>
+      </c>
+      <c r="C909" s="7" t="inlineStr">
+        <is>
+          <t>f452da9e</t>
+        </is>
+      </c>
+      <c r="D909" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-09 dev: add stop-frontend.ps1 + start.bat preflight 연동</t>
+        </is>
+      </c>
+      <c r="E909" s="7" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="F909" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="910">
+      <c r="A910" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B910" s="15" t="inlineStr">
+        <is>
+          <t>08:59</t>
+        </is>
+      </c>
+      <c r="C910" s="15" t="inlineStr">
+        <is>
+          <t>1ca2f201</t>
+        </is>
+      </c>
+      <c r="D910" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-09 frontend: 불량 탭 피드백 개선 — 부분 수량 복귀·부서 필터·KPI 카드 분리</t>
+        </is>
+      </c>
+      <c r="E910" s="15" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F910" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="911">
+      <c r="A911" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B911" s="7" t="inlineStr">
+        <is>
+          <t>09:23</t>
+        </is>
+      </c>
+      <c r="C911" s="7" t="inlineStr">
+        <is>
+          <t>a6874b75</t>
+        </is>
+      </c>
+      <c r="D911" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-09 frontend: 불량 탭 헤더 제거 + 뷰 전환 슬라이드 애니메이션</t>
+        </is>
+      </c>
+      <c r="E911" s="7" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F911" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="912">
+      <c r="A912" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B912" s="15" t="inlineStr">
+        <is>
+          <t>10:34</t>
+        </is>
+      </c>
+      <c r="C912" s="15" t="inlineStr">
+        <is>
+          <t>e9e169a5</t>
+        </is>
+      </c>
+      <c r="D912" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-09 frontend: 창고 지도 UX 개선 (열 클릭·자리 분할·슬롯 번호)</t>
+        </is>
+      </c>
+      <c r="E912" s="15" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F912" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="913">
+      <c r="A913" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B913" s="7" t="inlineStr">
+        <is>
+          <t>12:08</t>
+        </is>
+      </c>
+      <c r="C913" s="7" t="inlineStr">
+        <is>
+          <t>b88954e6</t>
+        </is>
+      </c>
+      <c r="D913" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-09 defect: 불량 탭 UX 개선 (카트 흐름·뒤로가기·필터 정리)</t>
+        </is>
+      </c>
+      <c r="E913" s="7" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="F913" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="914">
+      <c r="A914" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B914" s="15" t="inlineStr">
+        <is>
+          <t>12:17</t>
+        </is>
+      </c>
+      <c r="C914" s="15" t="inlineStr">
+        <is>
+          <t>d3440b9a</t>
+        </is>
+      </c>
+      <c r="D914" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-09 frontend: fix E2E test — update io-defect spec for hub 3-card flow</t>
+        </is>
+      </c>
+      <c r="E914" s="15" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F914" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="915">
+      <c r="A915" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B915" s="7" t="inlineStr">
+        <is>
+          <t>14:55</t>
+        </is>
+      </c>
+      <c r="C915" s="7" t="inlineStr">
+        <is>
+          <t>167f5dcb</t>
+        </is>
+      </c>
+      <c r="D915" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-09 defect: 격리 목록 UX 개선 — 출처 기본값·제목·배지·체크박스</t>
+        </is>
+      </c>
+      <c r="E915" s="7" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="F915" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="916">
+      <c r="A916" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B916" s="15" t="inlineStr">
+        <is>
+          <t>15:14</t>
+        </is>
+      </c>
+      <c r="C916" s="15" t="inlineStr">
+        <is>
+          <t>4e8d018a</t>
+        </is>
+      </c>
+      <c r="D916" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-09 defect: 창고 격리 → department='창고' 그룹 표시</t>
+        </is>
+      </c>
+      <c r="E916" s="15" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="F916" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="917">
+      <c r="A917" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B917" s="7" t="inlineStr">
+        <is>
+          <t>15:27</t>
+        </is>
+      </c>
+      <c r="C917" s="7" t="inlineStr">
+        <is>
+          <t>2c7b40fa</t>
+        </is>
+      </c>
+      <c r="D917" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-09 defect: 창고 담당자 격리 목록 기본 스코프 전체로 변경</t>
+        </is>
+      </c>
+      <c r="E917" s="7" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="F917" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="918">
+      <c r="A918" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B918" s="15" t="inlineStr">
+        <is>
+          <t>08:04</t>
+        </is>
+      </c>
+      <c r="C918" s="15" t="inlineStr">
+        <is>
+          <t>4282e7f5</t>
+        </is>
+      </c>
+      <c r="D918" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-10 defect: 처리 패널 재설계 + 부서 접기/펼치기 UX</t>
+        </is>
+      </c>
+      <c r="E918" s="15" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="F918" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="919">
+      <c r="A919" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B919" s="7" t="inlineStr">
+        <is>
+          <t>08:05</t>
+        </is>
+      </c>
+      <c r="C919" s="7" t="inlineStr">
+        <is>
+          <t>ff39db2f</t>
+        </is>
+      </c>
+      <c r="D919" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-10 backend: unquarantine reason_category optional 처리</t>
+        </is>
+      </c>
+      <c r="E919" s="7" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F919" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="920">
+      <c r="A920" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B920" s="15" t="inlineStr">
+        <is>
+          <t>08:34</t>
+        </is>
+      </c>
+      <c r="C920" s="15" t="inlineStr">
+        <is>
+          <t>34870c58</t>
+        </is>
+      </c>
+      <c r="D920" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-10 test: io-defect E2E 안정화 — 정상복귀 제출 셀렉터 모호성 해소</t>
+        </is>
+      </c>
+      <c r="E920" s="15" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="F920" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="921">
+      <c r="A921" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B921" s="7" t="inlineStr">
+        <is>
+          <t>08:51</t>
+        </is>
+      </c>
+      <c r="C921" s="7" t="inlineStr">
+        <is>
+          <t>30c4b20b</t>
+        </is>
+      </c>
+      <c r="D921" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-10 docs: 주간보고 6/7~6/10 갱신</t>
+        </is>
+      </c>
+      <c r="E921" s="7" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="F921" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
2026-06-11 docs: 주간보고 06/06~06/11 전사공유 버전 + 개발현황 5/30~6/11 행 추가
- 주간보고 6/6~6/11: 전사공유용 도입문 추가, 효과 중심 톤으로 전면 재작성
- generate_devlog.py: 5/30~6/5·6/6~6/11 주차 행 추가로 개발현황 요약 시트 업데이트
- 접속 안내 "(사내망 연결 환경에서만 접속 가능합니다.)" 추가

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_attic/docs/개발현황.xlsx
+++ b/_attic/docs/개발현황.xlsx
@@ -570,7 +570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E56"/>
+  <dimension ref="A1:E57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="67.25" customWidth="1" min="1" max="1"/>
@@ -616,7 +616,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>920건 (회사 기간 670건)</t>
+          <t>964건 (회사 기간 670건)</t>
         </is>
       </c>
     </row>
@@ -628,7 +628,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>326건 (평일 야간·주말·휴가 시간 커밋)</t>
+          <t>333건 (평일 야간·주말·휴가 시간 커밋)</t>
         </is>
       </c>
     </row>
@@ -1991,20 +1991,54 @@
               <color rgb="00000000"/>
               <sz val="10"/>
             </rPr>
-            <t>■■</t>
+            <t>■■■■■■</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00ED7D31"/>
+              <sz val="10"/>
+            </rPr>
+            <t>■■■</t>
           </r>
           <r>
             <rPr>
               <color rgb="00000000"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">  (4)</t>
+            <t xml:space="preserve">  (19)</t>
           </r>
         </is>
       </c>
     </row>
+    <row r="57" ht="18" customHeight="1">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">2026-06-11  </t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+              <sz val="10"/>
+            </rPr>
+            <t>■■■■■■■■■■■■■■</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">  (29)</t>
+          </r>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="54">
+  <mergeCells count="55">
     <mergeCell ref="A30:E30"/>
     <mergeCell ref="A39:E39"/>
     <mergeCell ref="A34:E34"/>
@@ -2036,6 +2070,7 @@
     <mergeCell ref="A12:E12"/>
     <mergeCell ref="A50:E50"/>
     <mergeCell ref="A26:E26"/>
+    <mergeCell ref="A57:E57"/>
     <mergeCell ref="A42:E42"/>
     <mergeCell ref="A33:E33"/>
     <mergeCell ref="A47:E47"/>
@@ -2070,7 +2105,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2330,7 +2365,7 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>사내 시연 + 양식 정비 + 운영 정책 맞춤 + 사번 audit</t>
+          <t>사내 시연 + 양식 정비 + 운영 정책 맞춤 + 사번 감사</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
@@ -2351,6 +2386,59 @@
       </c>
       <c r="D12" s="7" t="n">
         <v>177</v>
+      </c>
+    </row>
+    <row r="13" ht="113.4" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-30 ~ 06-05</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>코드 품질 + 아키텍처 정비</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>수량 정수 전용(IntQuantity) 아키텍처 정비 — 입력 422·출력·내부 일관화
+ItemCode → mes_code 전면 리네임 완료
+legacy → mes 폴더 개명 (프론트엔드 라우트 전면 재정리)
+클린코드 Phase 1 — schemas/ 분리·_tx_filters·README 정비
+디자인 일관성 정비 — Pretendard 실로딩 확인·EmptyState 중복 정리
+useToggleSet 훅으로 토글 중복 12개 통합, React Query 패널 3종 이관
+Admin Depts/Employees 하위 분리, 불량 처리 재설계 착수</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="n">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="14" ht="129.6" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-06 ~ 06-11</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>모바일 구성 + 불량 처리 재설계</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>불량 처리 패널 전면 재설계 + KPI 2개로 압축·부서 범위 명시
+격리 목록 기본 스코프 '전체' 전환·배지·체크박스 UX 개선
+창고 지도 열 클릭·슬롯 번호·박스 편집 기능 — 실사용 기반 마련
+직원별 품목 순서 커스터마이징 (드래그 재정렬·초기화)
+모바일 핵심 화면 구성 — 하단 탭 4개 + 더보기 시트
+모바일 불량 처리 카트 방식 전환 — 다품목 일괄 처리 가능
+io_preview·창고지도·불량 카트 단위 테스트 신설
+코드 품질 정비 — verify_local 전체 통과 확인</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="n">
+        <v>88</v>
       </c>
     </row>
   </sheetData>
@@ -4495,7 +4583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D47"/>
+  <dimension ref="A1:D48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5592,24 +5680,49 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="54" customHeight="1">
+    <row r="47" ht="67.5" customHeight="1">
       <c r="A47" s="7" t="inlineStr">
         <is>
           <t>2026-06-10</t>
         </is>
       </c>
       <c r="B47" s="7" t="n">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="C47" s="8" t="inlineStr">
         <is>
           <t>2026-06-10 defect: 처리 패널 재설계 + 부서 접기/펼치기 UX
 2026-06-10 backend: unquarantine reason_category optional 처리
 2026-06-10 test: io-defect E2E 안정화 — 정상복귀 제출 셀렉터 모호성 해소
-2026-06-10 docs: 주간보고 6/7~6/10 갱신</t>
+2026-06-10 docs: 주간보고 6/8~6/10 갱신
+2026-06-10 frontend: trim BACKEND_INTERNAL_URL — .env 공백/CRL</t>
         </is>
       </c>
       <c r="D47" s="7" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="67.5" customHeight="1">
+      <c r="A48" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B48" s="15" t="n">
+        <v>29</v>
+      </c>
+      <c r="C48" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-11 mobile: 하단 더보기 탭화·활성표시 강화 + 입출고 토스트 자동소멸
+2026-06-11 mobile: 불량 처리 데스크톱 정합 — 통합 처리 패널 모바일 신설
+2026-06-11 mobile: 입출고 저장슬롯 분리(손실 수정) + Step2 버튼 정합
+2026-06-11 mobile: 내역 상세 링크 날짜 자동 전환 + 뒤로가기 스택 pop
+2026-06-11 mobile: 내역 카드 최소 터치 높이(min-h-60) 보장</t>
+        </is>
+      </c>
+      <c r="D48" s="15" t="inlineStr">
         <is>
           <t>Frontend</t>
         </is>
@@ -5626,7 +5739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F921"/>
+  <dimension ref="A1:F965"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -35085,17 +35198,17 @@
       </c>
       <c r="B921" s="7" t="inlineStr">
         <is>
-          <t>08:51</t>
+          <t>08:55</t>
         </is>
       </c>
       <c r="C921" s="7" t="inlineStr">
         <is>
-          <t>30c4b20b</t>
+          <t>9cf2b98a</t>
         </is>
       </c>
       <c r="D921" s="8" t="inlineStr">
         <is>
-          <t>2026-06-10 docs: 주간보고 6/7~6/10 갱신</t>
+          <t>2026-06-10 docs: 주간보고 6/8~6/10 갱신</t>
         </is>
       </c>
       <c r="E921" s="7" t="inlineStr">
@@ -35104,6 +35217,1414 @@
         </is>
       </c>
       <c r="F921" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="922">
+      <c r="A922" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B922" s="15" t="inlineStr">
+        <is>
+          <t>09:07</t>
+        </is>
+      </c>
+      <c r="C922" s="15" t="inlineStr">
+        <is>
+          <t>d8eeaaa1</t>
+        </is>
+      </c>
+      <c r="D922" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-10 frontend: trim BACKEND_INTERNAL_URL — .env 공백/CRLF 로그인 먹통 방어</t>
+        </is>
+      </c>
+      <c r="E922" s="15" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F922" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="923">
+      <c r="A923" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B923" s="7" t="inlineStr">
+        <is>
+          <t>10:24</t>
+        </is>
+      </c>
+      <c r="C923" s="7" t="inlineStr">
+        <is>
+          <t>58141e34</t>
+        </is>
+      </c>
+      <c r="D923" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-10 warehouse: 박스 편집 UI + 재고 배치 시드</t>
+        </is>
+      </c>
+      <c r="E923" s="7" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="F923" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="924">
+      <c r="A924" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B924" s="15" t="inlineStr">
+        <is>
+          <t>10:37</t>
+        </is>
+      </c>
+      <c r="C924" s="15" t="inlineStr">
+        <is>
+          <t>2d03c451</t>
+        </is>
+      </c>
+      <c r="D924" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-10 defect: KPI 카드 결재대기·오늘처리 제거 (2개→격리중·1년이상만)</t>
+        </is>
+      </c>
+      <c r="E924" s="15" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="F924" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="925">
+      <c r="A925" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B925" s="7" t="inlineStr">
+        <is>
+          <t>11:17</t>
+        </is>
+      </c>
+      <c r="C925" s="7" t="inlineStr">
+        <is>
+          <t>b2d7d795</t>
+        </is>
+      </c>
+      <c r="D925" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-10 frontend: 불량 KPI 건 단위·부서범위 부제·필터 연동</t>
+        </is>
+      </c>
+      <c r="E925" s="7" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F925" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="926">
+      <c r="A926" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B926" s="15" t="inlineStr">
+        <is>
+          <t>11:17</t>
+        </is>
+      </c>
+      <c r="C926" s="15" t="inlineStr">
+        <is>
+          <t>ea571ec3</t>
+        </is>
+      </c>
+      <c r="D926" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-10 docs: 불량 피드백 5건 해결 반영 + 권동환 복귀일 정정</t>
+        </is>
+      </c>
+      <c r="E926" s="15" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="F926" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="927">
+      <c r="A927" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B927" s="7" t="inlineStr">
+        <is>
+          <t>13:39</t>
+        </is>
+      </c>
+      <c r="C927" s="7" t="inlineStr">
+        <is>
+          <t>8904d1cf</t>
+        </is>
+      </c>
+      <c r="D927" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-10 refactor: DesktopLegacyShell→MesShell 이름 정리 + 복귀 리뷰 준비 문서 (#31)</t>
+        </is>
+      </c>
+      <c r="E927" s="7" t="inlineStr">
+        <is>
+          <t>refactor</t>
+        </is>
+      </c>
+      <c r="F927" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="928">
+      <c r="A928" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B928" s="15" t="inlineStr">
+        <is>
+          <t>15:18</t>
+        </is>
+      </c>
+      <c r="C928" s="15" t="inlineStr">
+        <is>
+          <t>40ac636f</t>
+        </is>
+      </c>
+      <c r="D928" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-10 defect: reason_category 필수 검증 제거 (선택 필드로 전환)</t>
+        </is>
+      </c>
+      <c r="E928" s="15" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="F928" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="929">
+      <c r="A929" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B929" s="7" t="inlineStr">
+        <is>
+          <t>15:46</t>
+        </is>
+      </c>
+      <c r="C929" s="7" t="inlineStr">
+        <is>
+          <t>41da22bd</t>
+        </is>
+      </c>
+      <c r="D929" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-10 ux: 목록·테이블 줄 호버 하이라이트 일관 적용</t>
+        </is>
+      </c>
+      <c r="E929" s="7" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="F929" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="930">
+      <c r="A930" s="19" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B930" s="19" t="inlineStr">
+        <is>
+          <t>17:21</t>
+        </is>
+      </c>
+      <c r="C930" s="19" t="inlineStr">
+        <is>
+          <t>f7f0b5ae</t>
+        </is>
+      </c>
+      <c r="D930" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-10 docs: 모바일 벤치마킹 리서치 문서 추가</t>
+        </is>
+      </c>
+      <c r="E930" s="19" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="F930" s="21" t="inlineStr">
+        <is>
+          <t>근무 외</t>
+        </is>
+      </c>
+    </row>
+    <row r="931">
+      <c r="A931" s="19" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B931" s="19" t="inlineStr">
+        <is>
+          <t>22:15</t>
+        </is>
+      </c>
+      <c r="C931" s="19" t="inlineStr">
+        <is>
+          <t>90136f32</t>
+        </is>
+      </c>
+      <c r="D931" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-10 warehouse: 단품 입출고 판별 헬퍼 isSingleInlineSubType 추가</t>
+        </is>
+      </c>
+      <c r="E931" s="19" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="F931" s="21" t="inlineStr">
+        <is>
+          <t>근무 외</t>
+        </is>
+      </c>
+    </row>
+    <row r="932">
+      <c r="A932" s="19" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B932" s="19" t="inlineStr">
+        <is>
+          <t>22:15</t>
+        </is>
+      </c>
+      <c r="C932" s="19" t="inlineStr">
+        <is>
+          <t>f5e80f9e</t>
+        </is>
+      </c>
+      <c r="D932" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-10 mobile: 입출고 스캔-우선 동선 + 단품 인라인 폼</t>
+        </is>
+      </c>
+      <c r="E932" s="19" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="F932" s="21" t="inlineStr">
+        <is>
+          <t>근무 외</t>
+        </is>
+      </c>
+    </row>
+    <row r="933">
+      <c r="A933" s="19" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B933" s="19" t="inlineStr">
+        <is>
+          <t>22:15</t>
+        </is>
+      </c>
+      <c r="C933" s="19" t="inlineStr">
+        <is>
+          <t>16360a30</t>
+        </is>
+      </c>
+      <c r="D933" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-10 mobile: 주간보고 모바일 전용 뷰 신설</t>
+        </is>
+      </c>
+      <c r="E933" s="19" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="F933" s="21" t="inlineStr">
+        <is>
+          <t>근무 외</t>
+        </is>
+      </c>
+    </row>
+    <row r="934">
+      <c r="A934" s="19" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B934" s="19" t="inlineStr">
+        <is>
+          <t>22:16</t>
+        </is>
+      </c>
+      <c r="C934" s="19" t="inlineStr">
+        <is>
+          <t>d5b92afe</t>
+        </is>
+      </c>
+      <c r="D934" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-10 mobile: 창고지도 모바일 뷰 신설</t>
+        </is>
+      </c>
+      <c r="E934" s="19" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="F934" s="21" t="inlineStr">
+        <is>
+          <t>근무 외</t>
+        </is>
+      </c>
+    </row>
+    <row r="935">
+      <c r="A935" s="19" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B935" s="19" t="inlineStr">
+        <is>
+          <t>22:16</t>
+        </is>
+      </c>
+      <c r="C935" s="19" t="inlineStr">
+        <is>
+          <t>92517f6b</t>
+        </is>
+      </c>
+      <c r="D935" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-10 mobile: 하단 탭 4개로 축소 + 더보기 시트</t>
+        </is>
+      </c>
+      <c r="E935" s="19" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="F935" s="21" t="inlineStr">
+        <is>
+          <t>근무 외</t>
+        </is>
+      </c>
+    </row>
+    <row r="936">
+      <c r="A936" s="19" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B936" s="19" t="inlineStr">
+        <is>
+          <t>22:44</t>
+        </is>
+      </c>
+      <c r="C936" s="19" t="inlineStr">
+        <is>
+          <t>07d1d05d</t>
+        </is>
+      </c>
+      <c r="D936" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-10 defect: 해제 reason_memo 선택 허용 — E2E 불량 복귀 복구</t>
+        </is>
+      </c>
+      <c r="E936" s="19" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="F936" s="21" t="inlineStr">
+        <is>
+          <t>근무 외</t>
+        </is>
+      </c>
+    </row>
+    <row r="937">
+      <c r="A937" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B937" s="7" t="inlineStr">
+        <is>
+          <t>09:09</t>
+        </is>
+      </c>
+      <c r="C937" s="7" t="inlineStr">
+        <is>
+          <t>b6f0ebab</t>
+        </is>
+      </c>
+      <c r="D937" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-11 mobile: 하단 더보기 탭화·활성표시 강화 + 입출고 토스트 자동소멸</t>
+        </is>
+      </c>
+      <c r="E937" s="7" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="F937" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="938">
+      <c r="A938" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B938" s="15" t="inlineStr">
+        <is>
+          <t>09:09</t>
+        </is>
+      </c>
+      <c r="C938" s="15" t="inlineStr">
+        <is>
+          <t>3964a2d3</t>
+        </is>
+      </c>
+      <c r="D938" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-11 mobile: 불량 처리 데스크톱 정합 — 통합 처리 패널 모바일 신설</t>
+        </is>
+      </c>
+      <c r="E938" s="15" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="F938" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="939">
+      <c r="A939" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B939" s="7" t="inlineStr">
+        <is>
+          <t>09:10</t>
+        </is>
+      </c>
+      <c r="C939" s="7" t="inlineStr">
+        <is>
+          <t>43224017</t>
+        </is>
+      </c>
+      <c r="D939" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-11 mobile: 입출고 저장슬롯 분리(손실 수정) + Step2 버튼 정합</t>
+        </is>
+      </c>
+      <c r="E939" s="7" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="F939" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="940">
+      <c r="A940" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B940" s="15" t="inlineStr">
+        <is>
+          <t>09:12</t>
+        </is>
+      </c>
+      <c r="C940" s="15" t="inlineStr">
+        <is>
+          <t>b826e06f</t>
+        </is>
+      </c>
+      <c r="D940" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-11 mobile: 내역 상세 링크 날짜 자동 전환 + 뒤로가기 스택 pop</t>
+        </is>
+      </c>
+      <c r="E940" s="15" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="F940" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="941">
+      <c r="A941" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B941" s="7" t="inlineStr">
+        <is>
+          <t>09:12</t>
+        </is>
+      </c>
+      <c r="C941" s="7" t="inlineStr">
+        <is>
+          <t>8ab8e8bb</t>
+        </is>
+      </c>
+      <c r="D941" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-11 mobile: 내역 카드 최소 터치 높이(min-h-60) 보장</t>
+        </is>
+      </c>
+      <c r="E941" s="7" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="F941" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="942">
+      <c r="A942" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B942" s="15" t="inlineStr">
+        <is>
+          <t>09:13</t>
+        </is>
+      </c>
+      <c r="C942" s="15" t="inlineStr">
+        <is>
+          <t>1a6c8e6a</t>
+        </is>
+      </c>
+      <c r="D942" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-11 mobile: 대시보드 불량(DEFECT) 공정 필터 동작 복구</t>
+        </is>
+      </c>
+      <c r="E942" s="15" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="F942" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="943">
+      <c r="A943" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B943" s="7" t="inlineStr">
+        <is>
+          <t>09:17</t>
+        </is>
+      </c>
+      <c r="C943" s="7" t="inlineStr">
+        <is>
+          <t>31302638</t>
+        </is>
+      </c>
+      <c r="D943" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-11 mobile: 관리 드릴다운 단일컬럼 가드 + 메시지 배너 sticky</t>
+        </is>
+      </c>
+      <c r="E943" s="7" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="F943" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="944">
+      <c r="A944" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B944" s="15" t="inlineStr">
+        <is>
+          <t>09:18</t>
+        </is>
+      </c>
+      <c r="C944" s="15" t="inlineStr">
+        <is>
+          <t>c35bff1b</t>
+        </is>
+      </c>
+      <c r="D944" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-11 mobile: primitive 인라인 색 토큰화</t>
+        </is>
+      </c>
+      <c r="E944" s="15" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="F944" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="945">
+      <c r="A945" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B945" s="7" t="inlineStr">
+        <is>
+          <t>09:20</t>
+        </is>
+      </c>
+      <c r="C945" s="7" t="inlineStr">
+        <is>
+          <t>9949c33e</t>
+        </is>
+      </c>
+      <c r="D945" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-11 mobile: 알림 네비 탭 검증(딥링크 가드) + VALID_TAB_IDS 상수화</t>
+        </is>
+      </c>
+      <c r="E945" s="7" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="F945" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="946">
+      <c r="A946" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B946" s="15" t="inlineStr">
+        <is>
+          <t>09:23</t>
+        </is>
+      </c>
+      <c r="C946" s="15" t="inlineStr">
+        <is>
+          <t>1bd56575</t>
+        </is>
+      </c>
+      <c r="D946" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-11 mobile: 입출고 작성 중 섹션 이탈 가드</t>
+        </is>
+      </c>
+      <c r="E946" s="15" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="F946" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="947">
+      <c r="A947" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B947" s="7" t="inlineStr">
+        <is>
+          <t>09:25</t>
+        </is>
+      </c>
+      <c r="C947" s="7" t="inlineStr">
+        <is>
+          <t>afef8101</t>
+        </is>
+      </c>
+      <c r="D947" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-11 mobile: 입출고 서브탭(승인함·장바구니 등) 터치 타깃 44px 보장</t>
+        </is>
+      </c>
+      <c r="E947" s="7" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="F947" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="948">
+      <c r="A948" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B948" s="15" t="inlineStr">
+        <is>
+          <t>09:27</t>
+        </is>
+      </c>
+      <c r="C948" s="15" t="inlineStr">
+        <is>
+          <t>a5e8b76e</t>
+        </is>
+      </c>
+      <c r="D948" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-11 mobile: 입출고 인수인계 섹션 모바일 노출</t>
+        </is>
+      </c>
+      <c r="E948" s="15" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="F948" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="949">
+      <c r="A949" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B949" s="7" t="inlineStr">
+        <is>
+          <t>10:04</t>
+        </is>
+      </c>
+      <c r="C949" s="7" t="inlineStr">
+        <is>
+          <t>55f7aab5</t>
+        </is>
+      </c>
+      <c r="D949" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-11 mobile: 불량 격리·바로폐기 다품목 카트 모바일 신설(MobileDefectCartFlow)</t>
+        </is>
+      </c>
+      <c r="E949" s="7" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="F949" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="950">
+      <c r="A950" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B950" s="15" t="inlineStr">
+        <is>
+          <t>10:04</t>
+        </is>
+      </c>
+      <c r="C950" s="15" t="inlineStr">
+        <is>
+          <t>419a8d1a</t>
+        </is>
+      </c>
+      <c r="D950" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-11 mobile: 불량 허브 격리추가·바로폐기를 다품목 카트로 배선</t>
+        </is>
+      </c>
+      <c r="E950" s="15" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="F950" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="951">
+      <c r="A951" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B951" s="7" t="inlineStr">
+        <is>
+          <t>10:04</t>
+        </is>
+      </c>
+      <c r="C951" s="7" t="inlineStr">
+        <is>
+          <t>0d3be79d</t>
+        </is>
+      </c>
+      <c r="D951" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-11 mobile: 불량 화면 품목/모델 로드 + defaultSource(데스크톱 분리 패턴)</t>
+        </is>
+      </c>
+      <c r="E951" s="7" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="F951" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="952">
+      <c r="A952" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B952" s="15" t="inlineStr">
+        <is>
+          <t>10:04</t>
+        </is>
+      </c>
+      <c r="C952" s="15" t="inlineStr">
+        <is>
+          <t>8da005f1</t>
+        </is>
+      </c>
+      <c r="D952" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-11 mobile: DefectHubPanel 테스트 — 격리추가/바로폐기 카트 전환 검증</t>
+        </is>
+      </c>
+      <c r="E952" s="15" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="F952" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="953">
+      <c r="A953" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B953" s="7" t="inlineStr">
+        <is>
+          <t>10:49</t>
+        </is>
+      </c>
+      <c r="C953" s="7" t="inlineStr">
+        <is>
+          <t>37943d31</t>
+        </is>
+      </c>
+      <c r="D953" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-11 mobile: 관리 4섹션 크래시 수정 + 마스터-디테일 단일컬럼</t>
+        </is>
+      </c>
+      <c r="E953" s="7" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="F953" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="954">
+      <c r="A954" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B954" s="15" t="inlineStr">
+        <is>
+          <t>10:50</t>
+        </is>
+      </c>
+      <c r="C954" s="15" t="inlineStr">
+        <is>
+          <t>720114b4</t>
+        </is>
+      </c>
+      <c r="D954" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-11 mobile: 입출고 위저드 헤더가 셸 헤더 덮던 문제 수정</t>
+        </is>
+      </c>
+      <c r="E954" s="15" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="F954" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="955">
+      <c r="A955" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B955" s="7" t="inlineStr">
+        <is>
+          <t>10:52</t>
+        </is>
+      </c>
+      <c r="C955" s="7" t="inlineStr">
+        <is>
+          <t>0a5551d0</t>
+        </is>
+      </c>
+      <c r="D955" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-11 mobile: 입출고 섹션 탭 과밀 해소 — 모바일 가로 스크롤</t>
+        </is>
+      </c>
+      <c r="E955" s="7" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="F955" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="956">
+      <c r="A956" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B956" s="15" t="inlineStr">
+        <is>
+          <t>10:54</t>
+        </is>
+      </c>
+      <c r="C956" s="15" t="inlineStr">
+        <is>
+          <t>e4338316</t>
+        </is>
+      </c>
+      <c r="D956" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-11 mobile: 대시보드 생산가능 패널 칩↔자세히보기 겹침 수정</t>
+        </is>
+      </c>
+      <c r="E956" s="15" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="F956" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="957">
+      <c r="A957" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B957" s="7" t="inlineStr">
+        <is>
+          <t>10:56</t>
+        </is>
+      </c>
+      <c r="C957" s="7" t="inlineStr">
+        <is>
+          <t>de2cf545</t>
+        </is>
+      </c>
+      <c r="D957" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-11 mobile: 비율 폴리시 — 알림 시간 가독성·패널 폭 안전·카트 삭제 터치</t>
+        </is>
+      </c>
+      <c r="E957" s="7" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="F957" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="958">
+      <c r="A958" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B958" s="15" t="inlineStr">
+        <is>
+          <t>11:46</t>
+        </is>
+      </c>
+      <c r="C958" s="15" t="inlineStr">
+        <is>
+          <t>940e6c3f</t>
+        </is>
+      </c>
+      <c r="D958" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-11 mobile: 관리(admin) 화면을 모바일에서 제거</t>
+        </is>
+      </c>
+      <c r="E958" s="15" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="F958" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="959">
+      <c r="A959" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B959" s="7" t="inlineStr">
+        <is>
+          <t>11:57</t>
+        </is>
+      </c>
+      <c r="C959" s="7" t="inlineStr">
+        <is>
+          <t>9850f4ff</t>
+        </is>
+      </c>
+      <c r="D959" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-11 mobile: 입출고 Step4 라인 세로글자 수정 — IoLineRow 반응형</t>
+        </is>
+      </c>
+      <c r="E959" s="7" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="F959" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="960">
+      <c r="A960" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B960" s="15" t="inlineStr">
+        <is>
+          <t>12:01</t>
+        </is>
+      </c>
+      <c r="C960" s="15" t="inlineStr">
+        <is>
+          <t>0eb4b52a</t>
+        </is>
+      </c>
+      <c r="D960" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-11 mobile: 폴리시 — 불량 BOM 트리 품목명 줄바꿈 + 입출고 picker 필터 폭</t>
+        </is>
+      </c>
+      <c r="E960" s="15" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="F960" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="961">
+      <c r="A961" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B961" s="7" t="inlineStr">
+        <is>
+          <t>12:44</t>
+        </is>
+      </c>
+      <c r="C961" s="7" t="inlineStr">
+        <is>
+          <t>2b46b2ff</t>
+        </is>
+      </c>
+      <c r="D961" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-11 mobile: 비율 정리 — 불량 피커 필터·BOM 하위트리 폭·내역 캘린더 셀높이 반응형</t>
+        </is>
+      </c>
+      <c r="E961" s="7" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="F961" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="962">
+      <c r="A962" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B962" s="15" t="inlineStr">
+        <is>
+          <t>14:05</t>
+        </is>
+      </c>
+      <c r="C962" s="15" t="inlineStr">
+        <is>
+          <t>9f8a434b</t>
+        </is>
+      </c>
+      <c r="D962" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-11 mobile: 불량 화면이 화면 폭을 꽉 채우도록 수정 (w-full)</t>
+        </is>
+      </c>
+      <c r="E962" s="15" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="F962" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="963">
+      <c r="A963" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B963" s="7" t="inlineStr">
+        <is>
+          <t>15:04</t>
+        </is>
+      </c>
+      <c r="C963" s="7" t="inlineStr">
+        <is>
+          <t>147ac4e5</t>
+        </is>
+      </c>
+      <c r="D963" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-11 mobile: 품목 피커 목록이 화면 폭을 꽉 채우도록 colgroup 반응형화</t>
+        </is>
+      </c>
+      <c r="E963" s="7" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="F963" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="964">
+      <c r="A964" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B964" s="15" t="inlineStr">
+        <is>
+          <t>15:16</t>
+        </is>
+      </c>
+      <c r="C964" s="15" t="inlineStr">
+        <is>
+          <t>9c9c23d0</t>
+        </is>
+      </c>
+      <c r="D964" s="16" t="inlineStr">
+        <is>
+          <t>@ 2026-06-11 docs: ERD를 발표 스타일 HTML 문서로 추가</t>
+        </is>
+      </c>
+      <c r="E964" s="15" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="F964" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="965">
+      <c r="A965" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B965" s="7" t="inlineStr">
+        <is>
+          <t>15:32</t>
+        </is>
+      </c>
+      <c r="C965" s="7" t="inlineStr">
+        <is>
+          <t>cb357d2b</t>
+        </is>
+      </c>
+      <c r="D965" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-11 mobile: 원시 라벨·JSON 노출 정리 + 대시보드 현재고 우측정렬</t>
+        </is>
+      </c>
+      <c r="E965" s="7" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="F965" s="7" t="inlineStr">
         <is>
           <t>근무</t>
         </is>

</xml_diff>